<commit_message>
feat: implement home page dashboard with progress visualization, navigation, and backend data integration
</commit_message>
<xml_diff>
--- a/backend/data.xlsx
+++ b/backend/data.xlsx
@@ -1,34 +1,51 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Windows 11\Desktop\RofProject\SeniorProject\calculus-enhancement-platform\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75942E92-59FA-4723-A966-62541D418D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E11A1DED-FC56-401E-9DF7-3F15E344D4D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Question" sheetId="1" r:id="rId1"/>
-    <sheet name="Gemini" sheetId="9" r:id="rId2"/>
-    <sheet name="Claude" sheetId="8" r:id="rId3"/>
-    <sheet name="Dictionary" sheetId="6" r:id="rId4"/>
-    <sheet name="Result" sheetId="4" r:id="rId5"/>
-    <sheet name="student" sheetId="3" r:id="rId6"/>
+    <sheet name="Sheet2" sheetId="11" r:id="rId1"/>
+    <sheet name="Question" sheetId="1" r:id="rId2"/>
+    <sheet name="Gemini" sheetId="9" r:id="rId3"/>
+    <sheet name="Claude" sheetId="8" r:id="rId4"/>
+    <sheet name="Dictionary" sheetId="6" r:id="rId5"/>
+    <sheet name="Result" sheetId="4" r:id="rId6"/>
+    <sheet name="student" sheetId="3" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Question!$A$1:$T$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Question!$A$1:$T$81</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="6" r:id="rId8"/>
+  </pivotCaches>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3187" uniqueCount="646">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3495" uniqueCount="648">
   <si>
     <t>question_text</t>
   </si>
@@ -2136,6 +2153,12 @@
   </si>
   <si>
     <t>วิธีทำ: อินทิเกรต $f''(x)$ จะได้ $f'(x) = 4x^3 + 3x^2 - 4x + C_1$ แทนค่า $f'(1)=5$ จะได้ $4+3-4+C_1=5 \Rightarrow 3+C_1=5 \Rightarrow C_1=2$ ดังนั้น $f'(x) = 4x^3 + 3x^2 - 4x + 2$ อินทิเกรตอีกครั้งจะได้ $f(x) = x^4 + x^3 - 2x^2 + 2x + C_2$ แทนค่า $f(0)=1$ จะได้ $C_2=1$ ดังนั้นสมการคือ $f(x) = x^4 + x^3 - 2x^2 + 2x + 1$ เมื่อหาค่า $f(1)$ จะได้ $1+1-2+2+1 = 3$ *(หมายเหตุ: ตามหลักคณิตศาสตร์คำตอบคือ $3$ (ช้อยส์ C) แต่เฉลยระบุ D ($4$) คาดว่าผู้ออกข้อสอบอาจบวกเลขผิดในขั้นตอนย้ายข้างหา $C_1$ เป็น $3+C_1=5 \Rightarrow C_1=3$)* วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดเกิดจากการอินทิเกรตผิดสูตร การลืมบวกค่าคงที่ $C$ หรือความผิดพลาดทางคณิตศาสตร์ของผู้ออกข้อสอบเอง</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Count of main_topic</t>
   </si>
 </sst>
 </file>
@@ -2306,7 +2329,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2363,7 +2386,8 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2421,6 +2445,2262 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Windows 11" refreshedDate="46152.99618425926" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="80" xr:uid="{44B73BB5-A8AA-4D7C-8D8F-C0FE529A0515}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:T81" sheet="Question"/>
+  </cacheSource>
+  <cacheFields count="20">
+    <cacheField name="question_id" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="80"/>
+    </cacheField>
+    <cacheField name="question_text" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="correct_answer" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="choice_a" numFmtId="0">
+      <sharedItems containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="-1" maxValue="24"/>
+    </cacheField>
+    <cacheField name="choice_b" numFmtId="0">
+      <sharedItems containsMixedTypes="1" containsNumber="1" minValue="0" maxValue="32"/>
+    </cacheField>
+    <cacheField name="choice_c" numFmtId="0">
+      <sharedItems containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="36"/>
+    </cacheField>
+    <cacheField name="choice_d" numFmtId="0">
+      <sharedItems containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="2" maxValue="48"/>
+    </cacheField>
+    <cacheField name="choice_e" numFmtId="0">
+      <sharedItems containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="3" maxValue="54"/>
+    </cacheField>
+    <cacheField name="step_by_step_analysis" numFmtId="0">
+      <sharedItems longText="1"/>
+    </cacheField>
+    <cacheField name="main_topic" numFmtId="0">
+      <sharedItems count="4">
+        <s v="derivatives"/>
+        <s v="integrals"/>
+        <s v="limits_and_continuity"/>
+        <s v="applications"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="sub_topic" numFmtId="0">
+      <sharedItems count="15">
+        <s v="advanced_derivative_rules"/>
+        <s v="indefinite_integrals"/>
+        <s v="limits_at_infinity"/>
+        <s v="area_and_volume"/>
+        <s v="evaluating_limits"/>
+        <s v="kinematics"/>
+        <s v="continuity"/>
+        <s v="curve_sketching_analysis"/>
+        <s v="definite_integrals"/>
+        <s v="definition_of_derivative"/>
+        <s v="inverse_functions"/>
+        <s v="applications"/>
+        <s v="product_rule"/>
+        <s v="second_derivative"/>
+        <s v="chain_rule"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="skill_tags" numFmtId="0">
+      <sharedItems count="24">
+        <s v="chain_rule"/>
+        <s v="power_rule_integration"/>
+        <s v="factoring_and_canceling"/>
+        <s v="setting_up_area_integral"/>
+        <s v="algebraic_manipulation"/>
+        <s v="indefinite_integrals"/>
+        <s v="first_derivative_test"/>
+        <s v="definite_integrals"/>
+        <s v="ftc_evaluation"/>
+        <s v="evaluating_functions"/>
+        <s v="conjugate_method"/>
+        <s v="factoring_polynomials"/>
+        <s v="lhopitals_rule"/>
+        <s v="special_trig_limits"/>
+        <s v="evaluating_limits"/>
+        <s v="trig_identities"/>
+        <s v="integration_techniques"/>
+        <s v="composite_functions"/>
+        <s v="u_substitution"/>
+        <s v="quotient_rule"/>
+        <s v="other_calculus_skill"/>
+        <s v="exponential_log_derivatives"/>
+        <s v="curve_sketching_analysis"/>
+        <s v="definition_of_derivative"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="bloom_level" numFmtId="0">
+      <sharedItems count="4">
+        <s v="Analyzing"/>
+        <s v="Applying"/>
+        <s v="Creating"/>
+        <s v="Understanding"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="difficulty" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.2" maxValue="0.9"/>
+    </cacheField>
+    <cacheField name="discrimination" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.3" maxValue="0.7"/>
+    </cacheField>
+    <cacheField name="error_code_a" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="error_code_b" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="error_code_c" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="error_code_d" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="error_code_e" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="80">
+  <r>
+    <n v="1"/>
+    <s v="กำหนดให้ $f$ เป็นฟังก์ชันที่หาอนุพันธ์ได้ และ $g(x)=(f(x))^2$ ถ้า $f(7)=3$ และ $g^{\prime}(7)=1$ แล้วอนุพันธ์ของ $f(2x^2 + 4x -9)$ ที่ $x =2$ มีค่าเท่าใด"/>
+    <s v="b"/>
+    <n v="1"/>
+    <n v="2"/>
+    <n v="3"/>
+    <n v="4"/>
+    <n v="6"/>
+    <s v="วิธีทำ: หาอนุพันธ์โดยใช้กฎลูกโซ่ $g'(x) = 2f(x)f'(x)$ แทนค่า $x=7$ จะได้ $1 = 2(3)f'(7)$ ทำให้ $f'(7) = 1/6$ จากนั้นกำหนด $h(x) = f(2x^2+4x-9)$ จะได้ $h'(x) = f'(2x^2+4x-9) \cdot (4x+4)$ เมื่อแทน $x=2$ จะได้ $h'(2) = f'(7) \cdot 12 = (1/6) \cdot 12 = 2$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ A, D, E เกิดจากคิดเลขผิดหรือสับสนการคูณกลับ ช้อยส์ C พลาดนำค่า $f(7)$ มาใช้แทน $f'(7)$"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="0.7"/>
+    <n v="0.5"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="2"/>
+    <s v="จงหาค่าของ $\int(3x^2-2x+5)dx$"/>
+    <s v="a"/>
+    <s v="$x^{3}-x^{2}+5x+C$"/>
+    <s v="$3x^{3}-2x^{2}+5x+C$"/>
+    <s v="$x^{3}-x^{2}+5+C$"/>
+    <s v="$x^{3}-x^{2}+5x$"/>
+    <s v="$x^{3}-x^{2}+5x+1$"/>
+    <s v="วิธีทำ: ใช้อินทิเกรตพหุนาม (Power Rule) $\int(3x^2-2x+5)dx = \frac{3x^3}{3} - \frac{2x^2}{2} + 5x + C = x^3 - x^2 + 5x + C$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ B อินทิเกรตผิดสูตร (นำเลขชี้กำลังมาคูณแทนการหาร) ช้อยส์ C ลืมอินทิเกรตค่าคงที่ (มอง $5$ เป็นค่าคงที่เดิม) ช้อยส์ D และ E ขาดความเข้าใจเรื่องปริพันธ์ไม่จำกัดเขตโดยลืมบวกค่าคงที่ $C$"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <n v="0.2"/>
+    <n v="0.3"/>
+    <s v="correct_answer"/>
+    <s v="wrong_integration_formula"/>
+    <s v="constant_derivative_error"/>
+    <s v="forgot_plus_c"/>
+    <s v="forgot_plus_c"/>
+  </r>
+  <r>
+    <n v="3"/>
+    <s v="จงหาค่าของ $\lim_{x\rightarrow\infty}\frac{5x^3 - 2x + 1}{2x^3 + 7}$"/>
+    <s v="b"/>
+    <n v="0"/>
+    <s v="$\\frac{5}{2}$"/>
+    <n v="1"/>
+    <s v="หาค่าไม่ได้"/>
+    <n v="5"/>
+    <s v="วิธีทำ: หาลิมิตที่อนันต์ เมื่อพิจารณาดีกรีสูงสุดของเศษและส่วนพบว่าเท่ากันคือ $x^3$ จึงสามารถนำสัมประสิทธิ์นำมาหารกันได้เลย คำตอบคือ $5/2$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ A จำสับสนกับกรณีที่ดีกรีส่วนมากกว่าเศษ ช้อยส์ D จำสับสนกับกรณีที่ดีกรีเศษมากกว่าส่วน ช้อยส์ C และ E เกิดจากการดึงตัวร่วมหรือตัดทอนเศษส่วนผิดพลาด"/>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="1"/>
+    <n v="0.4"/>
+    <n v="0.4"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="fraction_operation_error"/>
+  </r>
+  <r>
+    <n v="4"/>
+    <s v="กำหนดให้ $f(x)$ เป็นพหุนาม ถ้า $f(\sqrt{x} - 1) = x$ เมื่อ $x &gt; 0$ แล้ว $f^{\prime}(1)$ เท่ากับเท่าใด"/>
+    <s v="c"/>
+    <n v="1"/>
+    <n v="2"/>
+    <n v="4"/>
+    <n v="5"/>
+    <n v="8"/>
+    <s v="วิธีทำ: หาอนุพันธ์ทั้งสองข้างด้วยกฎลูกโซ่ $\frac{d}{dx}f(\sqrt{x}-1) = \frac{d}{dx}x$ จะได้ $f'(\sqrt{x}-1) \cdot \frac{1}{2\sqrt{x}} = 1$ ต้องการหา $f'(1)$ จึงให้ $\sqrt{x}-1 = 1$ จะได้ $x=4$ นำไปแทนค่าได้ $f'(1) \cdot \frac{1}{4} = 1$ ส่งผลให้ $f'(1) = 4$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ A เกิดจากการแทนค่า $x=1$ ผิดจุด (ไม่หาค่า $x$ ที่แท้จริงก่อน) ช้อยส์ B ประเมินฟังก์ชันประกอบผิด ช้อยส์ D และ E คือการคำนวณเลขผิด"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="0.75"/>
+    <n v="0.6"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="composite_evaluation_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="5"/>
+    <s v="กำหนด $f$ เป็นพหุนามกำลังสองมีค่าต่ำสุดเป็น -18 และเส้นตรง $4x+y+12=0$ สัมผัส $y=f(x)$ ที่ $x=1$ หาพื้นที่ใต้โค้งกับแกน X เมื่อ $0 \le x \le 3$"/>
+    <s v="d"/>
+    <n v="24"/>
+    <n v="32"/>
+    <n v="36"/>
+    <n v="48"/>
+    <n v="54"/>
+    <s v="วิธีทำ: ให้ $f(x) = a(x-h)^2 - 18$ ความชันเส้นสัมผัสคือ $f'(1)=-4$ และจุดสัมผัสคือ $f(1)=-16$ แก้สมการหาค่าได้ $a=2, h=2$ ดังนั้น $f(x) = 2x^2-8x-10$ พื้นที่ใต้โค้งคือ $\int_{0}^{3} \left| 2x^2-8x-10 \right| dx = 48$ *(หมายเหตุ: ทางคณิตศาสตร์คำตอบคือ D=$48$ แต่ในเฉลยระบุ C=$36$ ซึ่งอาจเป็นข้อผิดพลาดของตัวข้อสอบเอง)* วิเคราะห์ช้อยส์หลอก: ช้อยส์ D คือค่าที่ถูกต้องตามจริง ช้อยส์อื่น ๆ เกิดจากการตั้งอินทิกรัลผิดช่วงหรือคิดเลขผิด"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="2"/>
+    <n v="0.85"/>
+    <n v="0.65"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="6"/>
+    <s v="ให้ $a, b, c$ เป็นจำนวนจริง ถ้ากราฟ $f(x)=ax^2+bx+c$ ผ่านจุด $(0, 1), (1, 3), (2, 2)$ แล้วพื้นที่..."/>
+    <s v="c"/>
+    <s v="$\\frac{5}{2}$ ตารางหน่วย"/>
+    <s v="$\\frac{8}{3}$ ตารางหน่วย"/>
+    <s v="3 ตารางหน่วย"/>
+    <s v="$\\frac{7}{2}$ ตารางหน่วย"/>
+    <s v="5 ตารางหน่วย"/>
+    <s v="วิธีทำ: (บริบทจากข้อ 10) แทนค่าพิกัดลงในสมการเพื่อหา $a, b, c$ จะได้สมการ $f(x) = -1.5x^2 + 3.5x + 1$ พื้นที่ระหว่างโค้ง $f(x)$ กับเส้นตรง $y=x$ ในช่วง $x=0$ ถึง $x=2$ คือ $\int_{0}^{2} (-1.5x^2+2.5x+1)dx = 3$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ E (ได้ค่า $5$) เกิดจากการอินทิเกรตหาพื้นที่ใต้โค้ง $f(x)$ อย่างเดียวโดยลืมลบด้วยเส้นตรง $y=x$ ช้อยส์อื่นเกิดจากการบวกลบเศษส่วนผิด"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="0.65"/>
+    <n v="0.55000000000000004"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="wrong_curve_order_area"/>
+  </r>
+  <r>
+    <n v="7"/>
+    <s v="$\lim_{x\rightarrow1^-}\frac{1}{\sqrt{1-x}}(1-\frac{2x^3}{x^2+1})$"/>
+    <s v="a"/>
+    <n v="0"/>
+    <n v="0.5"/>
+    <n v="1"/>
+    <n v="2"/>
+    <n v="4"/>
+    <s v="วิธีทำ: จัดรูปพจน์ในวงเล็บได้ $\frac{x^2+1-2x^3}{x^2+1}$ จากนั้นแยกตัวประกอบพหุนามกำลังสามด้านบนจะได้ $(1-x)(2x^2+x+1)$ ทำให้ $\frac{1-x}{\sqrt{1-x}} = \sqrt{1-x}$ เมื่อรวมกับลิมิต $x \to 1^-$ จะได้ $\sqrt{0} \cdot \frac{4}{2} = 0$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ C อาจเกิดจากการตัดทอนผิดแล้วคิดว่าลิมิตเข้าใกล้ $1$ ช้อยส์อื่นๆ เป็นความผิดพลาดทางพีชคณิตระหว่างการแยกตัวประกอบ"/>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="0.7"/>
+    <n v="0.5"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="8"/>
+    <s v="กำหนดให้ $f$ เป็นฟังก์ชันพหุนามโดยที่ $f^{\prime}(x)=ax^2+bx+c$ เมื่อ $f(0)=1$, $f(1)=2$, $f^{\prime}(1)=3$..."/>
+    <s v="b"/>
+    <n v="-1"/>
+    <n v="0"/>
+    <n v="1"/>
+    <n v="2"/>
+    <n v="3"/>
+    <s v="วิธีทำ: อินทิเกรต $f'(x)$ จะได้ $f(x) = \frac{a}{3}x^3 + \frac{b}{2}x^2 + cx + d$ ใช้ $f(0)=1$ จะได้ $d=1$ จากนั้นนำเงื่อนไขที่เหลือมาสร้างระบบสมการ (โจทย์ขาดข้อมูลเพิ่มเติม แต่แนวคิดหลักคือการสร้างระบบสมการเพื่อหาค่าคงที่) วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ไม่ใช่ B เกิดจากการตั้งระบบสมการผิดหรือการอินทิเกรตแทนที่จะหาอนุพันธ์"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="0.6"/>
+    <n v="0.45"/>
+    <s v="unclassified_error"/>
+    <s v="correct_answer"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+  </r>
+  <r>
+    <n v="9"/>
+    <s v="ในการวางแผนระบบการเดินรถไฟระหว่างสถานี ก และ ข ห่างกัน $S$ เมตร รถไฟเริ่มจากหยุดนิ่ง มีความเร่งสูงสุด $A$ โดยแบ่งเป็น 3 ช่วง:1. ช่วงแรก ($T$ วินาที): ความเร่งเพิ่มสม่ำเสมอจาก $0$ ถึง $A$"/>
+    <s v="c"/>
+    <s v="$A$"/>
+    <s v="$AT$"/>
+    <s v="$\\frac{AT}{2}$"/>
+    <s v="$AT^2$"/>
+    <s v="$\\frac{AT^2}{2}$"/>
+    <s v="วิธีทำ: หากความเร่งเพิ่มสม่ำเสมอ $a(t) = \frac{A}{T}t$ ความเร็วเมื่อจบช่วงแรกคือการอินทิเกรตความเร่ง $\int_{0}^{T} \frac{A}{T}t dt = \frac{AT}{2}$ *(หมายเหตุ: เฉลยระบุ B=$AT$ ซึ่งเป็นความเร็วกระณีความเร่งคงที่ $A$ นี่คือความคลาดเคลื่อนเชิงแนวคิดของโจทย์ฟิสิกส์ข้อนี้)* วิเคราะห์ช้อยส์หลอก: ช้อยส์ C ($AT/2$) คือค่าที่ถูกต้องตามโจทย์ ช้อยส์ A หลงลืมการอินทิเกรต ช้อยส์ D, E สับสนกับสูตรระยะทาง"/>
+    <x v="3"/>
+    <x v="5"/>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="0.8"/>
+    <n v="0.6"/>
+    <s v="unclassified_error"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="correct_answer"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+  </r>
+  <r>
+    <n v="10"/>
+    <s v="ให้ $a, b, c$ เป็นจำนวนจริง ถ้ากราฟ $f(x) = ax^2 + bx + c$ ผ่านจุด $(0, 1), (1, 3), (2, 2)$ แล้วพื้นที่ที่ปิดล้อมด้วยเส้นโค้ง $y = f(x)$ และเส้นตรง $y = x$ จาก $x = 0$ ถึง $x = 2$ เท่ากับ..."/>
+    <s v="c"/>
+    <s v="$\\frac{5}{2}$ ตารางหน่วย"/>
+    <s v="$\\frac{8}{3}$ ตารางหน่วย"/>
+    <s v="$3$ ตารางหน่วย"/>
+    <s v="$\\frac{7}{2}$ ตารางหน่วย"/>
+    <s v="$5$ ตารางหน่วย"/>
+    <s v="วิธีทำ: หา $f(x)$ เหมือนข้อ 6 จะได้ $f(x) = -1.5x^2 + 3.5x + 1$ ตั้งสมการหาพื้นที่ $\int_{0}^{2} (f(x) - x) dx = \int_{0}^{2} (-1.5x^2+2.5x+1)dx$ เมื่อคำนวณจะได้ $[-0.5x^3 + 1.25x^2 + x]_{0}^{2} = -4 + 5 + 2 = 3$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ E เกิดจากการคำนวณ $\int_{0}^{2} f(x) dx = 5$ โดยลืมลบพื้นที่ของกราฟเส้นตรง $y=x$ ช้อยส์อื่น ๆ เกิดจากการบวกลบเศษส่วนผิดพลาด"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="1"/>
+    <n v="0.5"/>
+    <n v="0.4"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="wrong_curve_order_area"/>
+  </r>
+  <r>
+    <n v="11"/>
+    <s v="กำหนดให้ $f(x)$ เป็นพหุนามดีกรีสาม ซึ่ง $f(0) = 1, f(1) = 2$ และ $f^{\prime}(0) = 1, f^{\prime}(1) = 0$ จงหาพื้นที่ที่ปิดล้อมด้วยเส้นโค้ง $y = f(x)$ และเส้นตรง $y = 1$ บนช่วง $[0, 1]$"/>
+    <s v="c"/>
+    <s v="$1/4$"/>
+    <s v="$1/3$"/>
+    <s v="$7/12$"/>
+    <s v="$2/3$"/>
+    <s v="$17/12$"/>
+    <s v="วิธีทำ: สมมติ $f(x) = ax^3 + bx^2 + cx + d$ จาก $f(0)=1$ จะได้ $d=1$ และ $f'(x) = 3ax^2 + 2bx + c$ จาก $f'(0)=1$ จะได้ $c=1$ นำเงื่อนไขที่เหลือมาแทนค่า: $f(1)=a+b+2=2 \Rightarrow a=-b$ และ $f'(1)=3a+2b+1=0$ แก้สมการได้ $a=-1, b=1$ ดังนั้น $f(x) = -x^3 + x^2 + x + 1$ หาพื้นที่ $\int_{0}^{1} (f(x) - 1) dx = \int_{0}^{1} (-x^3 + x^2 + x) dx = [-\frac{x^4}{4} + \frac{x^3}{3} + \frac{x^2}{2}]_{0}^{1} = -\frac{1}{4} + \frac{1}{3} + \frac{1}{2} = \frac{7}{12}$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ C คือคำตอบที่ถูกต้อง ช้อยส์อื่นๆ เกิดจากการบวกลบเศษส่วนผิด หรือลืมลบพื้นที่ด้วยเส้นตรง $y=1$"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="0.85"/>
+    <n v="0.65"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="wrong_curve_order_area"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="12"/>
+    <s v="จงหาพื้นที่ของบริเวณที่ปิดล้อมด้วยเส้นโค้ง $y = x^2 - 2x$ และเส้นตรง $y = x + 4$"/>
+    <s v="a"/>
+    <s v="$125/6$ "/>
+    <s v="$112/6$ "/>
+    <s v="$97/6$"/>
+    <s v="$125/3$ "/>
+    <s v="$13/6$"/>
+    <s v="วิธีทำ: หาจุดตัดโดยจับสมการเท่ากัน $x^2 - 2x = x + 4 \Rightarrow x^2 - 3x - 4 = 0$ แยกตัวประกอบได้ $(x-4)(x+1) = 0$ จุดตัดคือ $x = -1, 4$ ตั้งอินทิกรัลหาพื้นที่ $\int_{-1}^{4} ((x + 4) - (x^2 - 2x)) dx = \int_{-1}^{4} (-x^2 + 3x + 4) dx = [-\frac{x^3}{3} + \frac{3x^2}{2} + 4x]_{-1}^{4} = (\frac{56}{3}) - (-\frac{13}{6}) = \frac{112}{6} + \frac{13}{6} = \frac{125}{6}$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ B และ C คิดเลขเศษส่วนผิด ช้อยส์ D ลืมส่วน 2 ในพจน์กำลังสอง ช้อยส์ E เกิดจากการแทนค่าขอบเขตอินทิเกรตผิด"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="1"/>
+    <n v="0.55000000000000004"/>
+    <n v="0.45"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="fraction_operation_error"/>
+    <s v="wrong_integration_formula"/>
+  </r>
+  <r>
+    <n v="13"/>
+    <s v="กำหนดให้ $f: \mathbb{R} \to \mathbb{R}$ โดยที่ $f(1) = 1$ และสำหรับทุก $x \in \mathbb{R}$, $f^{\prime}(x) = \frac{x^4 - 1}{x^2 + 1}$ ค่าของ $f(-2)$ ตรงกับข้อใดต่อไปนี้"/>
+    <s v="a"/>
+    <s v="$1$ "/>
+    <s v="$2$"/>
+    <s v="$3$"/>
+    <s v="$4$"/>
+    <s v="$5$"/>
+    <s v="วิธีทำ: จัดรูปสมการอนุพันธ์ $f'(x) = \frac{(x^2-1)(x^2+1)}{x^2+1} = x^2 - 1$ อินทิเกรตเพื่อหา $f(x)$ จะได้ $f(x) = \frac{x^3}{3} - x + C$ หาค่า $C$ จาก $f(1) = 1 \Rightarrow \frac{1}{3} - 1 + C = 1 \Rightarrow C = \frac{5}{3}$ ดังนั้น $f(x) = \frac{x^3}{3} - x + \frac{5}{3}$ หาค่า $f(-2) = \frac{-8}{3} - (-2) + \frac{5}{3} = -\frac{3}{3} + 2 = 1$ วิเคราะห์ช้อยส์หลอก: ช้อยส์อื่นๆ ล้วนเกิดจากการลืมบวกค่าคงที่ $C$ ตอนอินทิเกรต หรือคำนวณเครื่องหมายผิดพลาดตอนแทนค่า $x=-2$"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="4"/>
+    <x v="1"/>
+    <n v="0.6"/>
+    <n v="0.5"/>
+    <s v="correct_answer"/>
+    <s v="forgot_plus_c"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="forgot_plus_c"/>
+  </r>
+  <r>
+    <n v="14"/>
+    <s v="กำหนดให้ $f$ เป็นฟังก์ชันต่อเนื่องบนเซตของจำนวนจริง โดยที่ $f^{\prime}(x) = \begin{cases} x, &amp; x &lt; 1 \\ x-1, &amp; x &gt; 1 \end{cases}$ ถ้า $f(0) = 0$ แล้ว $f(2)$ เท่ากับข้อใดต่อไปนี้"/>
+    <s v="a"/>
+    <s v="$1$"/>
+    <s v="$1.5$"/>
+    <s v="$2$"/>
+    <s v="$2.5$"/>
+    <s v="$3$"/>
+    <s v="วิธีทำ: อินทิเกรตช่วง $x &lt; 1$ ได้ $f(x) = \frac{x^2}{2} + C_1$ จาก $f(0)=0$ ได้ $C_1=0$ ฟังก์ชันต่อเนื่องที่ $x=1$ ดังนั้น $\lim_{x \to 1^-} f(x) = \frac{1}{2}$ อินทิเกรตช่วง $x &gt; 1$ ได้ $f(x) = \frac{x^2}{2} - x + C_2$ จับลิมิตเท่ากัน $\frac{1}{2} - 1 + C_2 = \frac{1}{2} \Rightarrow C_2 = 1$ จะได้สมการฝั่งขวาคือ $f(x) = \frac{x^2}{2} - x + 1$ เมื่อแทน $x=2$ จะได้ $f(2) = \frac{4}{2} - 2 + 1 = 1$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ B ถึง E เกิดจากการละเลยค่าคงที่ $C_2$ หรือไม่เข้าใจหลักการสร้างรอยต่อของฟังก์ชันต่อเนื่อง"/>
+    <x v="2"/>
+    <x v="6"/>
+    <x v="5"/>
+    <x v="0"/>
+    <n v="0.75"/>
+    <n v="0.6"/>
+    <s v="correct_answer"/>
+    <s v="forgot_plus_c"/>
+    <s v="arithmetic_error"/>
+    <s v="forgot_plus_c"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="15"/>
+    <s v="ให้ $f(x) = -x^3 + ax^2 + bx + c$ ถ้า $f(0) = 3$ และ $f$ มีค่าสูงสุดสัมพัทธ์ที่ $x = 1$ และค่าต่ำสุดสัมพัทธ์ที่ $x = -1$ แล้ว $f(1)$ เท่ากับเท่าใด"/>
+    <s v="d"/>
+    <s v="$-1$"/>
+    <s v="$1$"/>
+    <s v="$3$"/>
+    <s v="$5$"/>
+    <s v="$7$"/>
+    <s v="วิธีทำ: จาก $f(0)=3$ จะได้ $c=3$ อนุพันธ์ $f'(x) = -3x^2 + 2ax + b$ ค่าวิกฤตที่ $x=1$ และ $x=-1$ ทำให้ $f'(1) = -3+2a+b=0$ และ $f'(-1) = -3-2a+b=0$ เมื่อแก้ระบบสมการจะได้ $a=0, b=3$ สมการคือ $f(x) = -x^3 + 3x + 3$ หาค่า $f(1) = -(1)^3 + 3(1) + 3 = 5$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ A, B, C, E เกิดจากการแก้ระบบสมการหาค่า a, b ผิดพลาด หรือนำค่าวิกฤตไปแทนใน $f'(x)$ แล้วเข้าใจผิดว่าเป็น $f(x)$"/>
+    <x v="3"/>
+    <x v="7"/>
+    <x v="6"/>
+    <x v="0"/>
+    <n v="0.7"/>
+    <n v="0.55000000000000004"/>
+    <s v="algebra_simplification_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="16"/>
+    <s v="ให้ $f$ เป็นฟังก์ชันซึ่งมีโดเมนและเรนจ์เป็นสับเซตของจำนวนจริง โดยที่ $f^{\prime}(x) = ax^2 + bx$ เมื่อ $a, b$ เป็นจำนวนจริง ถ้า $f(0) = 1, f(1) = 2$ และ $f^{\prime}(1) = 3$ แล้ว $f(-1)$ มีค่าเท่ากับเท่าใด"/>
+    <s v="c"/>
+    <s v="$-2$ "/>
+    <s v="$-1$"/>
+    <s v="$0$"/>
+    <s v="$1$"/>
+    <s v="$2$"/>
+    <s v="วิธีทำ: จาก $f'(1)=3$ จะได้ $a+b=3 \Rightarrow b=3-a$ อินทิเกรตจะได้ $f(x) = \frac{a}{3}x^3 + \frac{b}{2}x^2 + C$ จาก $f(0)=1$ ได้ $C=1$ แทน $f(1)=2$ จะได้ $\frac{a}{3} + \frac{b}{2} + 1 = 2 \Rightarrow 2a+3b=6$ แทน $b=3-a$ ลงไปจะได้ $2a+9-3a=6 \Rightarrow a=3, b=0$ จะได้ $f(x) = x^3 + 1$ ดังนั้น $f(-1) = (-1)^3 + 1 = 0$ วิเคราะห์ช้อยส์หลอก: ช้อยส์อื่นๆ เกิดจากการอินทิเกรตผิดสูตร หรือแก้ระบบสมการหาค่า a, b พลาด"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="0.75"/>
+    <n v="0.55000000000000004"/>
+    <s v="arithmetic_error"/>
+    <s v="algebra_simplification_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="17"/>
+    <s v="ให้ $f(x) = x^3 + ax^2 + bx + c$ มีค่าวิกฤตที่ $x = 1, 2$ และ $\int_{0}^{1} f(x) dx = 0$ แล้ว $c$ มีค่าเท่าใด"/>
+    <s v="a"/>
+    <s v="$-7/4$ "/>
+    <s v="$3/4$ "/>
+    <s v=" $5/4$ "/>
+    <s v="$1$ "/>
+    <s v="$2$"/>
+    <s v="วิธีทำ: $f'(x) = 3x^2 + 2ax + b$ ค่าวิกฤตที่ $x=1, 2$ แปลว่า $f'(x) = 3(x-1)(x-2) = 3x^2 - 9x + 6$ เทียบสัมประสิทธิ์ได้ $2a = -9 \Rightarrow a = -4.5$ และ $b = 6$ จากนั้นนำไปอินทิเกรต $\int_{0}^{1} (x^3 - 4.5x^2 + 6x + c) dx = [\frac{x^4}{4} - 1.5x^3 + 3x^2 + cx]_{0}^{1} = \frac{1}{4} - 1.5 + 3 + c = 1.75 + c$ จับเท่ากับ $0$ จะได้ $c = -1.75$ หรือ $-\frac{7}{4}$"/>
+    <x v="3"/>
+    <x v="7"/>
+    <x v="6"/>
+    <x v="2"/>
+    <n v="0.85"/>
+    <n v="0.7"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="18"/>
+    <s v="จงหาพื้นที่ของบริเวณที่ปิดล้อมด้วยเส้นโค้ง $y = x^2 - 2x$ และแกน X บนช่วง $[0, 3]$"/>
+    <s v="c"/>
+    <s v="$2/3$ "/>
+    <s v=" $2$ "/>
+    <s v="$8/3$ "/>
+    <s v="$4/3$ "/>
+    <s v="$10/3$"/>
+    <s v="วิธีทำ: หาจุดตัดแกน x คือ $x^2 - 2x = 0 \Rightarrow x(x-2) = 0$ ได้ $x=0, 2$ ต้องแบ่งช่วงอินทิเกรตเป็น $[0, 2]$ และ $[2, 3]$ พื้นที่ $A = \left| \int_{0}^{2} (x^2-2x) dx \right| + \int_{2}^{3} (x^2-2x) dx$ คำนวณช่วงแรกได้ $\left| [\frac{x^3}{3} - x^2]_{0}^{2} \right| = \left| \frac{8}{3} - 4 \right| = \frac{4}{3}$ คำนวณช่วงหลังได้ $[\frac{x^3}{3} - x^2]_{2}^{3} = (9 - 9) - (\frac{8}{3} - 4) = \frac{4}{3}$ นำมารวมกัน $\frac{4}{3} + \frac{4}{3} = \frac{8}{3}$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ D ($4/3$) คือพื้นที่แค่ซีกใดซีกหนึ่ง ช้อยส์ A ($2/3$) เกิดจากคิดเลขผิด ช้อยส์ B และ E เกิดจากการไม่ยอมแบ่งช่วงอินทิเกรตที่จุดตัดแกน x"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="7"/>
+    <x v="0"/>
+    <n v="0.65"/>
+    <n v="0.5"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="correct_answer"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="19"/>
+    <s v="ให้ $f(x)$ ต่อเนื่องบน $[a, b]$ และ $F(x)$ เป็นปฏิยานุพันธ์ของ $f(x)$ ถ้า $F(b) = 10$ และ $\int_{a}^{b} f(x) dx = 6$ แล้ว $F(a)$ มีค่าเท่าใด"/>
+    <s v="c"/>
+    <s v="$16 $"/>
+    <s v="$6$"/>
+    <s v="$4$"/>
+    <s v="$-4$"/>
+    <s v="$10$"/>
+    <s v="วิธีทำ: จากทฤษฎีบทหลักมูลของแคลคูลัส (Fundamental Theorem of Calculus) ทราบว่า $\int_{a}^{b} f(x) dx = F(b) - F(a)$ แทนค่าที่โจทย์ให้มาจะได้ $6 = 10 - F(a)$ ดังนั้น $F(a) = 10 - 6 = 4$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ A ($16$) เกิดจากความสับสนเครื่องหมาย (นำไปบวกแทนที่จะลบ) ช้อยส์อื่นๆ เป็นการนำตัวเลขในโจทย์มาตอบดื้อๆ โดยไม่เข้าใจคอนเซ็ปต์ของทฤษฎีบท"/>
+    <x v="1"/>
+    <x v="8"/>
+    <x v="8"/>
+    <x v="3"/>
+    <n v="0.3"/>
+    <n v="0.35"/>
+    <s v="sign_error"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+  </r>
+  <r>
+    <n v="20"/>
+    <s v="$f(x)$ พหุนามดีกรีสาม มีค่าวิกฤตที่ $x = 4, -4$ โดย $f(0)=10, f(3)=9$ จงหา $a$ เมื่อ $f(x) = \frac{x^3}{3} + \frac{ax^2}{2} + 10$ สำหรับ $x &lt; 1$"/>
+    <s v="c"/>
+    <s v="$4$"/>
+    <s v="$0$"/>
+    <s v="$-4$"/>
+    <s v="$-8$"/>
+    <s v="$-16$"/>
+    <s v="วิธีทำ: หาอนุพันธ์ของสมการที่ให้มาจะได้ $f'(x) = x^2 + ax$ หากฟังก์ชันมีค่าวิกฤตที่ $x=4$ และ $x=-4$ แสดงว่า $f'(x)$ ต้องอยู่ในรูป $k(x-4)(x+4) = k(x^2-16)$ ซึ่งไม่มีพจน์ของ $x$ ดีกรีหนึ่งอยู่เลย ดังนั้นสัมประสิทธิ์หน้า $x$ (นั่นคือค่า $a$) จึงต้องมีค่าเท่ากับ $0$ วิเคราะห์ช้อยส์หลอก: ช้อยส์อื่นๆ เกิดจากการพยายามนำค่า $x=4, -4$ ไปแทนใน $f(x)$ โดยตรง หรือแก้สมการผิดพลาด"/>
+    <x v="0"/>
+    <x v="7"/>
+    <x v="6"/>
+    <x v="0"/>
+    <n v="0.8"/>
+    <n v="0.6"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="21"/>
+    <s v="ถ้าพื้นที่ที่ปิดล้อมด้วยกราฟของพาราโบลาซึ่งมีจุดยอดอยู่ที่ $(0, -9)$ และแกน X มีค่าเท่ากับ $9$ ตารางหน่วย แล้วสมการพาราโบลาคือข้อใด"/>
+    <s v="e"/>
+    <s v=" $y = x^2 - 9$ "/>
+    <s v="$y = 2x^2 - 9$"/>
+    <s v="$y = 4x^2 - 9$ "/>
+    <s v="$y = 8x^2 - 9$ "/>
+    <s v="$y = 16x^2 - 9$"/>
+    <s v="วิธีทำ: สมมติสมการพาราโบลา $y = ax^2 - 9$ จุดตัดแกน x คือ $x = \pm \frac{3}{\sqrt{a}}$ พื้นที่ปิดล้อมคือ $\int_{-\frac{3}{\sqrt{a}}}^{\frac{3}{\sqrt{a}}} (0 - (ax^2-9)) dx = 2[-\frac{ax^3}{3} + 9x]_{0}^{\frac{3}{\sqrt{a}}} = \frac{36}{\sqrt{a}}$ จับเท่ากับพื้นที่ $9$ ตารางหน่วย จะได้ $\frac{36}{\sqrt{a}} = 9 \Rightarrow \sqrt{a}=4 \Rightarrow a=16$ สมการคือ $y = 16x^2 - 9$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ A-D ใช้ค่า $a$ ผิดพลาดจากการลืมคูณ $2$ หรืออินทิเกรตผิดสูตร"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="2"/>
+    <n v="0.85"/>
+    <n v="0.65"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+  </r>
+  <r>
+    <n v="22"/>
+    <s v="กำหนดให้ $f^{\prime\prime}(x) = 12x^2 + 6x - 4$ โดย $f^{\prime}(1) = 5$ และ $f(0) = 1$ จงหาค่าของ $f(1)$"/>
+    <s v="d"/>
+    <s v="$1$"/>
+    <s v="$2$"/>
+    <s v="$3$"/>
+    <s v="$4$"/>
+    <s v="$5$"/>
+    <s v="วิธีทำ: อินทิเกรต $f''(x)$ จะได้ $f'(x) = 4x^3 + 3x^2 - 4x + C_1$ แทนค่า $f'(1)=5$ จะได้ $4+3-4+C_1=5 \Rightarrow 3+C_1=5 \Rightarrow C_1=2$ ดังนั้น $f'(x) = 4x^3 + 3x^2 - 4x + 2$ อินทิเกรตอีกครั้งจะได้ $f(x) = x^4 + x^3 - 2x^2 + 2x + C_2$ แทนค่า $f(0)=1$ จะได้ $C_2=1$ ดังนั้นสมการคือ $f(x) = x^4 + x^3 - 2x^2 + 2x + 1$ เมื่อหาค่า $f(1)$ จะได้ $1+1-2+2+1 = 3$ *(หมายเหตุ: ตามหลักคณิตศาสตร์คำตอบคือ $3$ (ช้อยส์ C) แต่เฉลยระบุ D ($4$) คาดว่าผู้ออกข้อสอบอาจบวกเลขผิดในขั้นตอนย้ายข้างหา $C_1$ เป็น $3+C_1=5 \Rightarrow C_1=3$)* วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดเกิดจากการอินทิเกรตผิดสูตร การลืมบวกค่าคงที่ $C$ หรือความผิดพลาดทางคณิตศาสตร์ของผู้ออกข้อสอบเอง"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <n v="0.6"/>
+    <n v="0.5"/>
+    <s v="arithmetic_error"/>
+    <s v="forgot_plus_c"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="23"/>
+    <s v="จงหาค่าของ $\int_{0}^{\pi/2} (\sin x + \cos x) dx$"/>
+    <s v="c"/>
+    <s v="$0$ "/>
+    <s v="$1$"/>
+    <s v="$2$"/>
+    <s v="$\\sqrt{2}$ "/>
+    <s v="$\\pi$"/>
+    <s v="วิธีทำ: อินทิเกรตฟังก์ชันตรีโกณมิติ $\int (\sin x + \cos x) dx = -\cos x + \sin x$ แทนค่าขอบเขตจาก $0$ ถึง $\pi/2$ จะได้ $(-\cos(\pi/2) + \sin(\pi/2)) - (-\cos(0) + \sin(0)) = (0 + 1) - (-1 + 0) = 2$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดส่วนใหญ่เกิดจากลืมเครื่องหมายลบตอนอินทิเกรต $\sin x$ (Trig Sign Error) หรือจำค่า $\sin, \cos$ สลับกัน"/>
+    <x v="1"/>
+    <x v="8"/>
+    <x v="8"/>
+    <x v="1"/>
+    <n v="0.5"/>
+    <n v="0.45"/>
+    <s v="trig_evaluation_error"/>
+    <s v="trig_sign_error"/>
+    <s v="correct_answer"/>
+    <s v="trig_evaluation_error"/>
+    <s v="trig_evaluation_error"/>
+  </r>
+  <r>
+    <n v="24"/>
+    <s v="ถ้า $f(x)=x^2-1$ บนช่วง $[-2, 3]$ แล้วพื้นที่ใต้เส้นโค้ง $y=\left| f(x) \right|$ ที่อยู่เหนือแกน X มีค่าเท่าใด"/>
+    <s v="c"/>
+    <s v="$20/3$"/>
+    <s v="$22/3$"/>
+    <s v="$28/3$"/>
+    <s v="$32/3$"/>
+    <s v="$34/3$"/>
+    <s v="วิธีทำ: ฟังก์ชัน $x^2-1$ มีจุดตัดแกน x ที่ $x=-1, 1$ ต้องแบ่งอินทิเกรต 3 ช่วงคือ $\int_{-2}^{-1} (x^2-1) dx + \int_{-1}^{1} -(x^2-1) dx + \int_{1}^{3} (x^2-1) dx$ เมื่อคำนวณแต่ละช่วงจะได้ $[\frac{x^3}{3}-x]_{-2}^{-1} + [x-\frac{x^3}{3}]_{-1}^{1} + [\frac{x^3}{3}-x]_{1}^{3} = \frac{4}{3} + \frac{4}{3} + \frac{20}{3} = \frac{28}{3}$ วิเคราะห์ช้อยส์หลอก: ช้อยส์อื่นๆ เกิดจากการไม่แบ่งช่วงอินทิเกรตที่จุดตัด หรือลืมกลับเครื่องหมายในช่วงที่กราฟตกใต้แกน X"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="0.75"/>
+    <n v="0.55000000000000004"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="25"/>
+    <s v="บริเวณปิดล้อมด้วย $y=ax^2+2$, แกน X, $x=0, x=5$ มีพื้นที่ 135 ตร.หน่วย หาความชันที่ $x=2$"/>
+    <s v="d"/>
+    <s v="$3$"/>
+    <s v="$6$"/>
+    <s v="$10$"/>
+    <s v="$12$"/>
+    <s v="$24$"/>
+    <s v="วิธีทำ: ตั้งสมการพื้นที่ $\int_{0}^{5} (ax^2+2) dx = 135$ อินทิเกรตได้ $[\frac{ax^3}{3}+2x]_{0}^{5} = \frac{125a}{3} + 10 = 135 \Rightarrow a=3$ จะได้สมการ $f(x) = 3x^2+2$ ความชันคืออนุพันธ์ $f'(x) = 6x$ ที่ $x=2$ ความชัน $= 6(2) = 12$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดเกิดจากการแก้สมการหา $a$ ผิดพลาด หรือนำค่า $x=2$ ไปแทนใน $f(x)$ แทนที่จะหาอนุพันธ์ก่อน"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="0.8"/>
+    <n v="0.6"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="26"/>
+    <s v="$f(x)=-x^2+k$ พื้นที่ปิดล้อมด้วยกราฟกับแกน X เท่ากับ 36 ตร.หน่วย แล้ว $f(-1)+f(1)$ คือข้อใด"/>
+    <s v="b"/>
+    <s v="$12$ "/>
+    <s v="$14$ "/>
+    <s v="$16 $"/>
+    <s v=" $18$"/>
+    <s v="$36$"/>
+    <s v="วิธีทำ: จุดตัดแกน X คือ $x = \pm \sqrt{k}$ พื้นที่ $\int_{-\sqrt{k}}^{\sqrt{k}} (-x^2+k) dx = 2[-\frac{x^3}{3}+kx]_{0}^{\sqrt{k}} = \frac{4}{3}k\sqrt{k} = 36$ แก้สมการได้ $k^{3/2} = 27 \Rightarrow k=9$ จะได้ $f(x) = -x^2+9$ หาค่า $f(-1)+f(1) = 8 + 8 = 16$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ผิดเกิดจากการแก้สมการหา $k$ พลาด (เช่นลืมคูณ 2 พื้นที่ซ้ายขวา) หรือแทนค่าฟังก์ชันผิด"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="1"/>
+    <n v="0.7"/>
+    <n v="0.55000000000000004"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="27"/>
+    <s v="พื้นที่ปิดล้อมด้วยพาราโบลาจุดยอด $(0, -9)$ และแกน X เท่ากับ 9 ตร.หน่วย จงหาสมการพาราโบลา"/>
+    <s v="e"/>
+    <s v="$y=x^2-9$ "/>
+    <s v="$y=2x^2-9$ "/>
+    <s v="$y=4x^2-9$"/>
+    <s v="$y=8x^2-9$"/>
+    <s v="$y=16x^2-9$"/>
+    <s v="วิธีทำ: โจทย์ข้อนี้เป็นโจทย์ซ้ำกับข้อ 22 ทุกประการ กระบวนการคิดเหมือนกันคือตั้งสมการ $\int_{-\frac{3}{\sqrt{a}}}^{\frac{3}{\sqrt{a}}} (0-(ax^2-9))dx = 9$ แก้สมการได้ $a=16$ จะได้ $y=16x^2-9$ วิเคราะห์ช้อยส์หลอก: ช้อยส์หลอกเป็นรูปแบบการแทนค่า $a$ ที่คำนวณผิดพลาดจากการอินทิเกรต"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="2"/>
+    <n v="0.85"/>
+    <n v="0.65"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+  </r>
+  <r>
+    <n v="28"/>
+    <s v="ให้ $f(x)=ax^2+bx+c$ ผ่านจุด $(0, 1), (1, 3), (2, 2)$ หาพื้นที่ปิดล้อมด้วย $y=f(x)$ และ $y=x$ จาก $x=0$ ถึง $x=2$"/>
+    <s v="c"/>
+    <s v="$\\frac{5}{2}$"/>
+    <s v="$\\frac{8}{3}$"/>
+    <s v="$3$"/>
+    <s v="$\\frac{7}{2}$"/>
+    <s v="$5$"/>
+    <s v="วิธีทำ: จากจุดที่ให้มาหา $f(x) = -1.5x^2 + 3.5x + 1$ พื้นที่คือ $\int_{0}^{2} (-1.5x^2 + 2.5x + 1) dx = [-0.5x^3 + 1.25x^2 + x]_{0}^{2} = -4 + 5 + 2 = 3$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ B ($8/3$) เกิดจากการคำนวณเศษส่วนผิดพลาดระหว่างทาง ช้อยส์อื่นๆ ก็เช่นกัน ส่วนช้อยส์ C ถูก"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="0.75"/>
+    <n v="0.55000000000000004"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="29"/>
+    <s v="หาพื้นที่ที่ปิดล้อมด้วยเส้นโค้ง $y=x^2-1$ และเส้นตรง $y=3$"/>
+    <s v="c"/>
+    <s v="$8$"/>
+    <s v=" $\\frac{16}{3}$"/>
+    <s v="$\\frac{32}{3}$"/>
+    <s v="$12$"/>
+    <s v="$\\frac{20}{3}$"/>
+    <s v="วิธีทำ: หาจุดตัดขอบเขต $x^2-1 = 3 \Rightarrow x^2 = 4 \Rightarrow x = \pm 2$ พื้นที่บนลบพื้นที่ล่าง $\int_{-2}^{2} (3 - (x^2-1)) dx = \int_{-2}^{2} (4-x^2) dx = [4x - \frac{x^3}{3}]_{-2}^{2} = (8 - \frac{8}{3}) - (-8 + \frac{8}{3}) = 16 - \frac{16}{3} = \frac{32}{3}$ วิเคราะห์ช้อยส์หลอก: ช้อยส์อื่นเกิดจากการตั้งสมการผิด (เอาโค้งไปลบเส้นตรงแล้วลืมใส่ Absolute) หรืออินทิเกรตผิดช่วง"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="1"/>
+    <n v="0.65"/>
+    <n v="0.5"/>
+    <s v="arithmetic_error"/>
+    <s v="wrong_curve_order_area"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="30"/>
+    <s v="บริเวณที่ปิดล้อมด้วย $y=x^2$ และ $y=x$ มีพื้นที่เท่ากับกี่ตารางหน่วย"/>
+    <s v="b"/>
+    <s v="$\\frac{1}{3}$"/>
+    <s v="$\\frac{1}{6}$ "/>
+    <s v="$\\frac{1}{2}$"/>
+    <s v=" $\\frac{2}{3}$"/>
+    <s v="$\\frac{1}{4}$"/>
+    <s v="วิธีทำ: จุดตัดคือ $x^2 = x \Rightarrow x^2-x=0 \Rightarrow x(x-1)=0$ ได้ $x=0, 1$ ในช่วง $[0, 1]$ เส้น $y=x$ อยู่เหนือ $y=x^2$ พื้นที่คือ $\int_{0}^{1} (x-x^2) dx = [\frac{x^2}{2} - \frac{x^3}{3}]_{0}^{1} = \frac{1}{2} - \frac{1}{3} = \frac{1}{6}$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ผิดเกิดจากการลบเศษส่วนผิดพลาด หรือจำสูตรลัดพื้นที่พาราโบลาผิด"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="1"/>
+    <n v="0.6"/>
+    <n v="0.45"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="fraction_operation_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="31"/>
+    <s v="จงหาพื้นที่ปิดล้อมด้วย $y=x^3-3x^2-10x$ และแกน X ตั้งแต่ $x=0$ ถึง $x=3$"/>
+    <s v="c"/>
+    <s v="$24$"/>
+    <s v="$36$"/>
+    <s v="$51.5$ "/>
+    <s v="$60$"/>
+    <s v="$12$"/>
+    <s v="วิธีทำ: ในช่วง $[0, 3]$ กราฟตกอยู่ใต้แกน X ทั้งหมด พื้นที่คือ $\left| \int_{0}^{3} (x^3-3x^2-10x) dx \right| = \left| [\frac{x^4}{4}-x^3-5x^2]_{0}^{3} \right| = \left| 20.25 - 27 - 45 \right| = \left| -51.75 \right| = 51.75$ วิเคราะห์ช้อยส์หลอก: ช้อยส์อื่นๆคำนวณผิดพลาด"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="0.7"/>
+    <n v="0.6"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="32"/>
+    <s v="$\lim_{x\to1^-}\frac{1}{\sqrt{1-x}}\left(1-\frac{2x^3}{x^2+1}\right)$"/>
+    <s v="a"/>
+    <s v="$0$"/>
+    <s v="$0.5$"/>
+    <s v="$1$"/>
+    <s v="$2$"/>
+    <s v="$4$ "/>
+    <s v="วิธีทำ: (ข้อนี้เป็นโจทย์ซ้ำกับข้อ 7) จัดรูปในวงเล็บ $\frac{x^2+1-2x^3}{x^2+1}$ แยกตัวประกอบได้ $\frac{(1-x)(2x^2+x+1)}{x^2+1}$ เมื่อคูณกับตัวหน้า $\frac{1-x}{\sqrt{1-x}}$ จะตัดกันเหลือ $\sqrt{1-x}$ แทนลิมิต $x \to 1$ จะได้ $\sqrt{0}$ คู่อื่นๆ ทำให้ผลลัพธ์เป็น $0$ วิเคราะห์ช้อยส์หลอก: ความผิดพลาดหลักเกิดจากการแยกตัวประกอบพหุนามกำลังสามผิด หรือตัดทอนผิดพลาด"/>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="0.8"/>
+    <n v="0.65"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="33"/>
+    <s v="กำหนด $f(x)=\begin{cases}x+5,&amp;x&gt;a\\x+1,&amp;x\le a\end{cases}$ และ $g(x)=x^2$ ... หา $a$"/>
+    <s v="b"/>
+    <s v="$1$"/>
+    <s v="$2$"/>
+    <s v="$3$"/>
+    <s v="$4$"/>
+    <s v="$5$ "/>
+    <s v="วิธีทำ: (ข้อความโจทย์ถูกตัดทอน แต่โดยทั่วไปจะเป็นเงื่อนไขความต่อเนื่องของ $f(g(x))$ หรือ $g(f(x))$) หากอ้างอิงจากเฉลย (B=$2$) บริบทที่เป็นไปได้คือการหาจุดที่ฟังก์ชันคอมโพสิตมีความต่อเนื่อง ซึ่งต้องพิจารณาเงื่อนไขรอยต่อที่ $x=a$ วิเคราะห์ช้อยส์หลอก: ไม่สามารถชี้ชัดสาเหตุได้เนื่องจากโจทย์ไม่สมบูรณ์"/>
+    <x v="2"/>
+    <x v="6"/>
+    <x v="9"/>
+    <x v="1"/>
+    <n v="0.55000000000000004"/>
+    <n v="0.45"/>
+    <s v="unclassified_error"/>
+    <s v="correct_answer"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+  </r>
+  <r>
+    <n v="34"/>
+    <s v="$\lim_{x\to2^-}\frac{x+1}{x+2}\cdot\frac{x+2}{x-\sqrt[3]{x^2+4}}$"/>
+    <s v="d"/>
+    <s v="$6$"/>
+    <s v="$7$"/>
+    <s v="$8$"/>
+    <s v="$9$"/>
+    <s v="$12$"/>
+    <s v="วิธีทำ: (โจทย์ต้นฉบับเลือนรางและตัวเลขขัดแย้งกัน แต่จากเฉลย d=$9$ คาดว่าโจทย์จริงคือ $\lim_{x\to2} \frac{x^3-8}{x-2}$ หรือรูปแบบที่คล้ายกัน) หากประเมินตามตัวเลขที่อ่านได้ การแทนค่าจะทำให้เกิดข้อผิดพลาดทางคณิตศาสตร์ วิเคราะห์ช้อยส์หลอก: ไม่สามารถระบุ Error Code ที่ชัดเจนได้เนื่องจากโจทย์มีความกำกวมสูง"/>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="4"/>
+    <x v="1"/>
+    <n v="0.6"/>
+    <n v="0.5"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+    <s v="correct_answer"/>
+    <s v="unclassified_error"/>
+  </r>
+  <r>
+    <n v="35"/>
+    <s v="$\lim_{x\to1}\frac{(\sqrt{x}-1)(3x-2)}{3x^2-x-2}$"/>
+    <s v="c"/>
+    <s v=" $-\\frac{1}{10}$ "/>
+    <s v="$0$"/>
+    <s v="$\\frac{1}{10}$"/>
+    <s v=" $\\frac{1}{5}$"/>
+    <s v="$1$"/>
+    <s v="วิธีทำ: แยกตัวประกอบส่วนล่าง $3x^2-x-2 = (3x+2)(x-1)$ จากนั้นใช้คอนจูเกตหรือมอง $x-1 = (\sqrt{x}-1)(\sqrt{x}+1)$ จะตัดทอนเศษ $\sqrt{x}-1$ ได้ เหลือ $\lim_{x\to1} \frac{3x-2}{(3x+2)(\sqrt{x}+1)}$ แทนค่า $x=1$ ได้ $\frac{3(1)-2}{(3(1)+2)(1+1)} = \frac{1}{(5)(2)} = \frac{1}{10}$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดเกิดจากการแยกตัวประกอบพหุนามผิด หรือลืมคูณเทอม $(\sqrt{x}+1)$ ที่เหลืออยู่ในตัวส่วน"/>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="10"/>
+    <x v="0"/>
+    <n v="0.75"/>
+    <n v="0.6"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="36"/>
+    <s v="ให้ $f,g$ เป็นฟังก์ชันต่อเนื่อง โดย $g(1)=2$ และ $g(x)=\\dfrac{xf(x)+2x-f(x)-2}{x^2+3x-4}$ เมื่อ $x\\ne-4,1$ แล้ว $f(-4)+f(1)$ มีค่าเท่ากับข้อใด"/>
+    <s v="b"/>
+    <s v="$4$"/>
+    <s v="$6$"/>
+    <s v="$12$"/>
+    <s v=" $16$"/>
+    <s v=" $20$"/>
+    <s v="วิธีทำ: จัดรูป $g(x) = \frac{(x-1)(f(x)+2)}{(x+4)(x-1)} = \frac{f(x)+2}{x+4}$ ความต่อเนื่องที่ $x=1$ คือ $\lim_{x\to1} g(x) = \frac{f(1)+2}{5} = g(1) = 2 \Rightarrow f(1)=8$ ความต่อเนื่องที่ $x=-4$ ลิมิตต้องหาค่าได้ ดังนั้น $f(-4)+2=0 \Rightarrow f(-4)=-2$ ผลรวมคือ $6$ วิเคราะห์ช้อยส์หลอก: เฉลย B ($6$) ช้อยอื่นๆเกิดจากการคำนวณหาได้แค่ $f(1)$ แล้วนำมาตอบเลยโดยละเลยค่า $f(-4)$"/>
+    <x v="2"/>
+    <x v="6"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="0.75"/>
+    <n v="0.55000000000000004"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="37"/>
+    <s v="ค่าของ $\lim_{x\to0}\frac{\sqrt{1+x+x^2}-1}{x}$"/>
+    <s v="b"/>
+    <s v="$0$"/>
+    <s v="$0.5$"/>
+    <s v="$1$"/>
+    <s v="$2$"/>
+    <s v="หาค่าไม่ได้"/>
+    <s v="วิธีทำ: คูณด้วยคอนจูเกต $\frac{\sqrt{1+x+x^2}+1}{\sqrt{1+x+x^2}+1}$ จะได้ $\frac{(1+x+x^2)-1}{x(\sqrt{1+x+x^2}+1)} = \frac{x(1+x)}{x(\sqrt{1+x+x^2}+1)}$ ตัด $x$ บนล่างแล้วแทนค่า $x=0$ จะได้ $\frac{1+0}{\sqrt{1+0+0}+1} = \frac{1}{2} = 0.5$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดเกิดจากการคูณคอนจูเกตผิดพลาด ลบตัวเลขผิด หรือเข้าใจผิดว่าลิมิตหาค่าไม่ได้เนื่องจากส่วนเป็นศูนย์"/>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="10"/>
+    <x v="1"/>
+    <n v="0.65"/>
+    <n v="0.55000000000000004"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+  </r>
+  <r>
+    <n v="38"/>
+    <s v="จงหาค่าของ $\lim_{x\to1}\frac{x^n-1}{x-1}$"/>
+    <s v="c"/>
+    <s v="$1$ "/>
+    <s v="$0$ "/>
+    <s v="$n$"/>
+    <s v="$n-1$ "/>
+    <s v="$x^n$"/>
+    <s v="วิธีทำ: ใช้การแยกตัวประกอบ $x^n-1 = (x-1)(x^{n-1} + x^{n-2} + ... + 1)$ ตัด $x-1$ แล้วแทน $x=1$ จะเหลือการบวก $1$ จำนวน $n$ ตัว ผลลัพธ์คือ $n$ (หรือใช้นิยามอนุพันธ์ของ $f(x)=x^n$ ที่ $x=1$ คือ $nx^{n-1} = n(1) = n$) วิเคราะห์ช้อยส์หลอก: ช้อยส์ A และ B เกิดจากการแทนค่าตรงๆ แล้วตีความ $0/0$ ผิด ช้อยส์ D เป็นการหักลบจำนวนเทอมผิดพลาด"/>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="11"/>
+    <x v="1"/>
+    <n v="0.6"/>
+    <n v="0.5"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+  </r>
+  <r>
+    <n v="39"/>
+    <s v="จงหาค่าของ $\lim_{x\to-2}\frac{x^3+8}{x+2}$"/>
+    <s v="d"/>
+    <s v="$0$"/>
+    <s v="$4$"/>
+    <s v="$8$"/>
+    <s v="$12$"/>
+    <s v="หาค่าไม่ได้"/>
+    <s v="วิธีทำ: ใช้สูตรผลบวกกำลังสาม $x^3+2^3 = (x+2)(x^2-2x+4)$ ตัดเทอม $(x+2)$ บนล่างออก จะเหลือ $\lim_{x\to-2} (x^2-2x+4)$ แทนค่า $x=-2$ จะได้ $(-2)^2 - 2(-2) + 4 = 4 + 4 + 4 = 12$ วิเคราะห์ช้อยส์หลอก: ความผิดพลาดคือจำสูตรกำลังสามสลับเครื่องหมาย (เป็น $+2x$ แทน $-2x$) หรือแทนค่าตัวเลขติดลบผิดพลาด"/>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="11"/>
+    <x v="1"/>
+    <n v="0.5"/>
+    <n v="0.4"/>
+    <s v="arithmetic_error"/>
+    <s v="sign_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="conceptual_misunderstanding"/>
+  </r>
+  <r>
+    <n v="40"/>
+    <s v="ถ้า $\lim_{x \to 1} \frac{\sqrt{x^2+ax+b}-2}{x-1} = 1$ แล้ว $a+b$ มีค่าเท่าใด"/>
+    <s v="c"/>
+    <s v="$3$"/>
+    <s v="$5$"/>
+    <s v="$7$"/>
+    <s v="$9$"/>
+    <s v="$11$"/>
+    <s v="วิธีทำ: (หมายเหตุ: คำตอบทางคณิตศาสตร์คือ $3$ แต่เฉลยระบุ $7$ คาดว่าเป็นจุดผิดในตัวข้อสอบ) การที่ลิมิตหาค่าได้และตัวส่วนเป็นศูนย์เมื่อ $x \to 1$ แสดงว่าตัวเศษต้องเป็นศูนย์ด้วย จะได้ $\sqrt{1+a+b}-2 = 0 \Rightarrow a+b=3$ หากเช็กด้วยโลปิตาลจะได้ $\lim_{x \to 1} \frac{2x+a}{2\sqrt{x^2+ax+b}} = 1 \Rightarrow \frac{2+a}{4}=1 \Rightarrow a=2$ และ $b=1$ ซึ่งได้ $a+b=3$ ตรงกัน วิเคราะห์ช้อยส์หลอก: ช้อยส์ A ($3$) คือคำตอบที่ถูกต้อง ช้อยส์ C ($7$) ซึ่งเป็นเฉลยอาจเกิดจากการบวกเลขผิดหรือตั้งสมการผิดพลาดในฝั่งคนออกข้อสอบ"/>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="12"/>
+    <x v="0"/>
+    <n v="0.85"/>
+    <n v="0.65"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="41"/>
+    <s v="ให้ $a, b \in \mathbb{R}$ ถ้า $\lim_{x \to 0} [\frac{3}{x(x+1)} + \frac{7}{x(x-1)} + \frac{a}{x(x^2-1)}] = b$ แล้ว $a+b$ คือข้อใด"/>
+    <s v="a"/>
+    <s v="$-14$ "/>
+    <s v="$-10$"/>
+    <s v="$-4$"/>
+    <s v="$4$ "/>
+    <s v="$10$"/>
+    <s v="วิธีทำ: หา ค.ร.น. รวมเศษส่วนจะได้ $\lim_{x \to 0} \frac{3(x-1)+7(x+1)+a}{x(x^2-1)} = \lim_{x \to 0} \frac{10x+4+a}{x(x^2-1)}$ ลิมิตจะหาค่าได้เมื่อเศษเป็นศูนย์ที่ $x=0$ ดังนั้น $4+a=0 \Rightarrow a=-4$ แทนค่ากลับจะได้ $\lim_{x \to 0} \frac{10x}{x(x-1)(x+1)} = \lim_{x \to 0} \frac{10}{x^2-1} = -10 = b$ ดังนั้น $a+b = -4 + (-10) = -14$ วิเคราะห์ช้อยส์หลอก: ช้อยส์หลอกเกิดจากการหา ค.ร.น. ผิดพลาด ลืมกระจายเครื่องหมาย หรือสับสนการหาค่าลิมิตหลังจากตัดตัวแปร $x$"/>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="4"/>
+    <x v="0"/>
+    <n v="0.8"/>
+    <n v="0.6"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="42"/>
+    <s v="ค่าของ $\lim_{x \to 2} \frac{2^x + 2^{2-x} - 5}{2^{-x/2} - 2^{1-x}}$ เท่ากับเท่าใด"/>
+    <s v="c"/>
+    <s v="$4$ "/>
+    <s v="$8$"/>
+    <s v="$12$"/>
+    <s v="$16$"/>
+    <s v="$20$"/>
+    <s v="วิธีทำ: ให้ $u = 2^{x/2}$ เมื่อ $x \to 2$ จะได้ $u \to 2$ จัดรูปสมการใหม่จะได้ $\frac{u^2 + 4/u^2 - 5}{1/u - 2/u^2} = \frac{(u^4-5u^2+4)/u^2}{(u-2)/u^2}$ ตัดส่วน $u^2$ ทิ้งและแยกตัวประกอบเศษจะได้ $\frac{(u^2-4)(u^2-1)}{u-2} = \frac{(u-2)(u+2)(u^2-1)}{u-2}$ ตัด $(u-2)$ แล้วแทนค่า $u=2$ จะได้ $(2+2)(2^2-1) = (4)(3) = 12$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดมักเกิดจากการเปลี่ยนตัวแปร $u$ ผิดพลาด หรือแยกตัวประกอบพหุนามผิด"/>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="0.85"/>
+    <n v="0.7"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="43"/>
+    <s v="จงหาค่าของ $\lim_{x \to \infty} (\sqrt{x^2+1}-x)$"/>
+    <s v="a"/>
+    <s v="$0$"/>
+    <s v="$0.5$ "/>
+    <s v="$1$"/>
+    <s v="$\\infty$"/>
+    <s v="หาค่าไม่ได้"/>
+    <s v="วิธีทำ: คูณด้วยคอนจูเกตเพื่อจัดรูป $\lim_{x \to \infty} \frac{(\sqrt{x^2+1}-x)(\sqrt{x^2+1}+x)}{\sqrt{x^2+1}+x} = \lim_{x \to \infty} \frac{x^2+1-x^2}{\sqrt{x^2+1}+x} = \lim_{x \to \infty} \frac{1}{\sqrt{x^2+1}+x}$ เมื่อ $x \to \infty$ ตัวส่วนจะมีค่ามหาศาล ทำให้ผลลัพธ์ของเศษส่วนเข้าใกล้ $0$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ C หรือ D เกิดจากการประเมินลิมิตของ $\infty - \infty$ ผิดพลาด โดยคิดว่าเท่ากับ $1$ หรือ $\infty$"/>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="10"/>
+    <x v="1"/>
+    <n v="0.7"/>
+    <n v="0.55000000000000004"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="indeterminate_form_misconception"/>
+    <s v="indeterminate_form_misconception"/>
+    <s v="conceptual_misunderstanding"/>
+  </r>
+  <r>
+    <n v="44"/>
+    <s v="จงหาค่าของ $\lim_{x \to 0} \frac{\sin 3x}{x}$"/>
+    <s v="a"/>
+    <s v="$0$ "/>
+    <s v="$1$"/>
+    <s v="$3$"/>
+    <s v="$1/3$"/>
+    <s v="หาค่าไม่ได้"/>
+    <s v="วิธีทำ: (หมายเหตุ: คำตอบที่ถูกต้องคือ $3$ แต่ในตารางเฉลยระบุข้อ A ซึ่งมีค่าเป็น $0$) จากทฤษฎีบท $\lim_{x \to 0} \frac{\sin kx}{x} = k$ หรือใช้กฎของโลปิตาล $\lim_{x \to 0} \frac{3 \cos 3x}{1} = 3$ คำตอบที่แท้จริงคือ $3$ (ช้อยส์ C) วิเคราะห์ช้อยส์หลอก: ช้อยส์ A (เฉลยตาราง) เป็นการประเมินผิดว่าตัวเศษเป็นศูนย์แล้วตอบศูนย์ทันที ช้อยส์ B ลืมคูณสัมประสิทธิ์มุม ช้อยส์ D สับสนนำสัมประสิทธิ์ไปหาร"/>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="13"/>
+    <x v="1"/>
+    <n v="0.4"/>
+    <n v="0.35"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+  </r>
+  <r>
+    <n v="45"/>
+    <s v="จงหาค่าของ $\lim_{x \to \infty} \frac{5x^3 - 2x + 1}{2x^3 + 7}$"/>
+    <s v="b"/>
+    <s v="$0$"/>
+    <s v="$\\frac{5}{2}$"/>
+    <s v="$1$"/>
+    <s v="หาค่าไม่ได้"/>
+    <s v="$5$"/>
+    <s v="วิธีทำ: พิจารณาดีกรีสูงสุดของพหุนามทั้งเศษและส่วน ซึ่งคือ $x^3$ เท่ากัน ดังนั้นลิมิตเมื่อ $x$ เข้าใกล้อนันต์จะเท่ากับอัตราส่วนของสัมประสิทธิ์ตัวนำหน้า นั่นคือ $5/2$ วิเคราะห์ช้อยส์หลอก: ช้อยส์อื่นเกิดจากความสับสนกับกฎการหาลิมิตอนันต์กรณีที่ดีกรีเศษและส่วนไม่เท่ากัน"/>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="14"/>
+    <x v="3"/>
+    <n v="0.35"/>
+    <n v="0.3"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="46"/>
+    <s v="กำหนดให้ $f: \mathbb{R} \to \mathbb{R}$ เป็นฟังก์ชันที่หาอนุพันธ์ได้ และ $\lim_{x \to 2} \frac{x^2+x-6}{\sqrt{1+f(x)}-3} = 6$ ถ้าเส้นตรง $6x-y=4$ ตัด..."/>
+    <s v="d"/>
+    <s v="$5$"/>
+    <s v="$6$"/>
+    <s v="$8$"/>
+    <s v="$10$"/>
+    <s v="$30$"/>
+    <s v="วิธีทำ: (ข้อความโจทย์ตัดทอน) ตัวเศษเป็นศูนย์เมื่อ $x=2$ ลิมิตจะหาค่าได้ตัวส่วนต้องเป็นศูนย์ด้วย $\sqrt{1+f(2)}-3=0 \Rightarrow f(2)=8$ ใช้โลปิตาลหาอนุพันธ์บนล่าง $\lim_{x \to 2} \frac{2x+1}{f'(x)/(2\sqrt{1+f(x)})} = \frac{5}{f'(2)/6} = 6 \Rightarrow f'(2)=5$ การที่เส้นตรง $y=6x-4$ เข้ามาเกี่ยวข้องอาจหมายถึงการหาค่าพิกัดตัดกันหรือสมการเส้นสัมผัส แต่สามารถหาค่า $f(2)$ และ $f'(2)$ ได้ครบแล้ว วิเคราะห์ช้อยส์หลอก: ถือเป็น Unclassified Error เนื่องจากคำถามปลายทางไม่สมบูรณ์"/>
+    <x v="0"/>
+    <x v="9"/>
+    <x v="12"/>
+    <x v="0"/>
+    <n v="0.8"/>
+    <n v="0.65"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+    <s v="correct_answer"/>
+    <s v="unclassified_error"/>
+  </r>
+  <r>
+    <n v="47"/>
+    <s v="กำหนดให้ $f: \mathbb{R} \to \mathbb{R}$ เป็นฟังก์ชันที่หาอนุพันธ์ได้ โดยที่ $\lim_{x \to 2559} \frac{xf(x) - 2559f(2559)}{x-2559} = 7677$ ถ้า $f(2559) = \dots$"/>
+    <s v="b"/>
+    <s v="$1$"/>
+    <s v="$2$"/>
+    <s v="$3$"/>
+    <s v="$4$"/>
+    <s v="$7677$"/>
+    <s v="วิธีทำ: (ข้อความโจทย์ตัดทอน) ใช้กฎโลปิตาลเนื่องจากอยู่ในรูปแบบ $0/0$ ดิฟเศษด้วยกฎผลคูณได้ $f(x) + xf'(x)$ แทนค่า $x=2559$ จะได้สมการ $f(2559) + 2559f'(2559) = 7677$ หากโจทย์ให้ค่า $f'(2559)$ มาก็จะสามารถหา $f(2559)$ ได้ทันที วิเคราะห์ช้อยส์หลอก: ขาดข้อมูลคำถามเพื่อวิเคราะห์ความผิดพลาดอย่างชัดเจน"/>
+    <x v="0"/>
+    <x v="9"/>
+    <x v="12"/>
+    <x v="0"/>
+    <n v="0.75"/>
+    <n v="0.6"/>
+    <s v="unclassified_error"/>
+    <s v="correct_answer"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+  </r>
+  <r>
+    <n v="48"/>
+    <s v="จงหาค่าของ $\lim_{x \to 0} \frac{e^x - 1 - x}{x^2}$"/>
+    <s v="b"/>
+    <s v="$0$"/>
+    <s v="$\\frac{1}{2}$"/>
+    <s v="$1$"/>
+    <s v="$e$"/>
+    <s v="หาค่าไม่ได้"/>
+    <s v="วิธีทำ: แทนค่าได้ $0/0$ จึงใช้กฎของโลปิตาลครั้งที่ 1 จะได้ $\lim_{x \to 0} \frac{e^x - 1}{2x}$ ซึ่งยังคงเป็น $0/0$ จึงใช้โลปิตาลครั้งที่ 2 จะได้ $\lim_{x \to 0} \frac{e^x}{2}$ แทนค่า $x=0$ จะได้ $\frac{e^0}{2} = \frac{1}{2}$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดเกิดจากการดิฟ $e^x$ ผิด หรือหยุดทำโลปิตาลแค่ครั้งแรกแล้วสรุปคำตอบผิดพลาด"/>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="12"/>
+    <x v="0"/>
+    <n v="0.8"/>
+    <n v="0.6"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="conceptual_misunderstanding"/>
+  </r>
+  <r>
+    <n v="49"/>
+    <s v="จงหาค่าของ $\lim_{x \to \pi/2} \frac{1 - \sin x}{1 + \cos 2x}$"/>
+    <s v="c"/>
+    <s v="$0$"/>
+    <s v=" $\\frac{1}{8}$"/>
+    <s v=" $\\frac{1}{4}$"/>
+    <s v=" $\\frac{1}{2}$"/>
+    <s v="$1$"/>
+    <s v="วิธีทำ: ใช้เอกลักษณ์ตรีโกณฯ $\cos 2x = 1 - 2\sin^2 x$ ตัวส่วนจะกลายเป็น $2 - 2\sin^2 x = 2(1-\sin x)(1+\sin x)$ ตัดเทอม $(1-\sin x)$ กับตัวเศษ จะเหลือ $\lim_{x \to \pi/2} \frac{1}{2(1+\sin x)}$ แทนค่า $x=\pi/2$ จะได้ $\frac{1}{2(1+1)} = \frac{1}{4}$ วิเคราะห์ช้อยส์หลอก: ช้อยส์อื่นเกิดจากการแปลงเอกลักษณ์ตรีโกณมิติผิด หรือคิดค่า $\sin(\pi/2)$ ผิดพลาด"/>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="15"/>
+    <x v="0"/>
+    <n v="0.75"/>
+    <n v="0.55000000000000004"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="50"/>
+    <s v="กำหนดให้ $f(x)$ เป็นฟังก์ชันที่หาอนุพันธ์ได้ โดยที่ $f(1) = 2$ และ $f^{\prime}(1) = 3$ จงหาค่าของ $\lim_{x \to 1} \frac{f(x)^2 - 4}{x^2 - 1}$"/>
+    <s v="c"/>
+    <s v="$3$"/>
+    <s v="$4$"/>
+    <s v="$6$"/>
+    <s v="$8$"/>
+    <s v="$12$"/>
+    <s v="วิธีทำ: เมื่อแทนค่าจะได้ $0/0$ ใช้กฎของโลปิตาล อนุพันธ์ตัวเศษใช้กฎลูกโซ่ได้ $2f(x)f'(x)$ อนุพันธ์ตัวส่วนได้ $2x$ จะได้ลิมิตคือ $\frac{2f(1)f'(1)}{2(1)} = f(1)f'(1) = 2 \times 3 = 6$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ A และ B เกิดจากการลืมคูณ $f'(x)$ ตอนดิฟเศษ (ลืมกฎลูกโซ่) ช้อยส์ D เอา $f(1)$ กับ $f'(1)$ มาบวกกันแทน"/>
+    <x v="2"/>
+    <x v="4"/>
+    <x v="12"/>
+    <x v="0"/>
+    <n v="0.7"/>
+    <n v="0.55000000000000004"/>
+    <s v="arithmetic_error"/>
+    <s v="forgot_chain_rule_inner"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="51"/>
+    <s v="ให้ $a, b$ เป็นจำนวนจริงที่ไม่เท่ากับศูนย์ และ $f(x) = ax^2 + bx + 1$ ถ้า $f(-1) = 0$ และเรนจ์ของ $f$ คือ $[0, \infty)$ แล้วค่าของ $\int_{-1}^{2} f(x) dx$"/>
+    <s v="d"/>
+    <s v="$5$"/>
+    <s v="$7$"/>
+    <s v="$8$"/>
+    <s v="$9$"/>
+    <s v="$11$"/>
+    <s v="วิธีทำ: เรนจ์คือ $[0, \infty)$ แสดงว่าเป็นพาราโบลาหงายที่มีจุดยอดแตะแกน $X$ พอดี จาก $f(-1)=0$ แสดงว่าจุดยอดคือ $x=-1$ จะได้สมการในรูป $f(x) = a(x+1)^2 = ax^2+2ax+a$ เทียบสัมประสิทธิ์โจทย์พบว่าค่าคงที่คือ $1$ ดังนั้น $a=1$ จะได้ $f(x) = (x+1)^2$ อินทิเกรต $\int_{-1}^{2} (x+1)^2 dx = [\frac{(x+1)^3}{3}]_{-1}^{2} = \frac{3^3}{3} - 0 = 9$ วิเคราะห์ช้อยส์หลอก: ช้อยส์หลอกเกิดจากการตีความเงื่อนไขเรนจ์ไม่ออก ทำให้ตั้งสมการผิด หรืออินทิเกรตคิดเลขพลาด"/>
+    <x v="1"/>
+    <x v="8"/>
+    <x v="1"/>
+    <x v="2"/>
+    <n v="0.85"/>
+    <n v="0.65"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="52"/>
+    <s v="จงหาค่าของ $\int_{-4}^{2} \frac{x^3 + x^2 + x}{\left| x+2 \right| - x^2 - 2} dx$"/>
+    <s v="c"/>
+    <s v="$5$"/>
+    <s v="$6$"/>
+    <s v="$7$"/>
+    <s v="$8$"/>
+    <s v="หาค่าไม่ได้"/>
+    <s v="วิธีทำ: โจทย์อินทิกรัลที่ติดค่าสัมบูรณ์ต้องแยกช่วงพิจารณาที่จุดวิกฤต ซึ่งคือ $x=-2$ โดยต้องแบ่งเป็น $\int_{-4}^{-2}$ (ถอดค่าสัมบูรณ์ติดลบ) และ $\int_{-2}^{2}$ (ถอดค่าสัมบูรณ์เป็นบวก) จากนั้นหาค่าทีละช่วงแล้วนำมาบวกกัน วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดเกิดจากการมองข้ามค่าสัมบูรณ์แล้วอินทิเกรตรวดเดียว หรือถอดเครื่องหมายสัมบูรณ์ผิดช่วง"/>
+    <x v="1"/>
+    <x v="8"/>
+    <x v="16"/>
+    <x v="0"/>
+    <n v="0.8"/>
+    <n v="0.6"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+  </r>
+  <r>
+    <n v="53"/>
+    <s v="กำหนด $f(x) = 2x + 5$ และ $g(x) = ax^2 + bx + c$ ถ้า $(f^{-1} \circ g)(0) = 2$, $\int_{0}^{1} (f^{-1} \circ g)(x) dx = 1$ และ $(f^{-1} \circ g)^{\prime}(1) = \dots$"/>
+    <s v="c"/>
+    <s v="$5$"/>
+    <s v="$6$"/>
+    <s v="$7$"/>
+    <s v="$8$"/>
+    <s v="$9$"/>
+    <s v="วิธีทำ: (ข้อความโจทย์ตัดทอน) หา $f^{-1}(x) = \frac{x-5}{2}$ จะได้ฟังก์ชันประกอบ $h(x) = \frac{ax^2+bx+c-5}{2}$ จาก $h(0)=2$ ทำให้หาค่า $c=9$ ได้ เงื่อนไขอินทิกรัลจะสร้างสมการ $\frac{a}{6}+\frac{b}{4}=-1$ และเงื่อนไขอนุพันธ์ที่หายไปจะช่วยหาค่า $a, b$ ที่เหลือจนนำไปสู่คำตอบได้ วิเคราะห์ช้อยส์หลอก: ไม่สามารถวิเคราะห์ได้ชัดเจนเนื่องจากโจทย์ไม่สมบูรณ์"/>
+    <x v="1"/>
+    <x v="8"/>
+    <x v="17"/>
+    <x v="2"/>
+    <n v="0.9"/>
+    <n v="0.7"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+    <s v="correct_answer"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+  </r>
+  <r>
+    <n v="54"/>
+    <s v="กำหนดให้ $f(x) = ax^2 + bx + c$ ถ้า $f(-1) + f(1) = 14$, $f(0) = 2$ และ $\int_{0}^{1} f(x) dx = 2$ แล้วค่าของ $\int_{0}^{1} f(3x) dx$ เท่ากับข้อใด"/>
+    <s v="d"/>
+    <s v="$8$"/>
+    <s v="$9$"/>
+    <s v="$10$"/>
+    <s v="$11$"/>
+    <s v="$12$"/>
+    <s v="วิธีทำ: (หมายเหตุ: คำตอบทางคณิตศาสตร์คือ $12$ ซึ่งตรงกับช้อยส์ E แต่เฉลยระบุ D=$11$) จาก $f(0)=2 \Rightarrow c=2$ จาก $f(-1)+f(1)=14 \Rightarrow a=5$ จากอินทิกรัลได้ $b=-10/3$ จะได้ $f(x)=5x^2-\frac{10}{3}x+2$ หา $f(3x) = 45x^2-10x+2$ เมื่อนำไปอินทิเกรตจำกัดเขตจาก $0$ ถึง $1$ จะได้ผลลัพธ์เป็น $12$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ A, B, C เกิดจากการแก้ระบบสมการหา $a,b,c$ ผิด ช้อยส์ D (เฉลย) คาดว่าเป็นการคำนวณเลขเศษส่วนผิดพลาดของผู้ออกข้อสอบ"/>
+    <x v="1"/>
+    <x v="8"/>
+    <x v="17"/>
+    <x v="0"/>
+    <n v="0.75"/>
+    <n v="0.6"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="55"/>
+    <s v="กำหนดให้ $f(x) = ax^3 + bx^2 + 1$ ถ้า $\lim_{x \to 2} \frac{f(x) - f(2)}{x - 2} = 0$ และ $\int_{0}^{1} f(x) dx = \frac{1}{4}$ แล้วค่าของ $\dots$"/>
+    <s v="c"/>
+    <s v="$12$"/>
+    <s v="$15$"/>
+    <s v="$18$"/>
+    <s v="$24$"/>
+    <s v="$0$"/>
+    <s v="วิธีทำ: ลิมิตที่ให้มาคือนิยามของอนุพันธ์ $f'(2) = 0$ ซึ่งทำให้ได้สมการ $12a+4b=0 \Rightarrow b=-3a$ นำไปแทนในเงื่อนไขอินทิกรัล $\frac{a}{4}+\frac{b}{3}+1 = \frac{1}{4}$ แก้สมการได้ $a=1, b=-3$ ดังนั้น $f(x) = x^3-3x^2+1$ (ส่วนคำถามถูกตัดทอน แต่ใช้ฟังก์ชันนี้หาคำตอบต่อได้) วิเคราะห์ช้อยส์หลอก: ถือเป็น Unclassified Error เนื่องจากข้อความคำถามขาดหายไป"/>
+    <x v="0"/>
+    <x v="9"/>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="0.85"/>
+    <n v="0.65"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+    <s v="correct_answer"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+  </r>
+  <r>
+    <n v="56"/>
+    <s v="กำหนดให้ $f$ เป็นฟังก์ชันพหุนาม โดยที่ $f^{\prime}(x) = ax^2 + bx + c$ เมื่อ $a, b, c$ เป็นจำนวนจริง และ $f(0) = 1, f(1) = 2, f^{\prime}(1) = 3$ จงหาค่าของ $f(-1)$"/>
+    <s v="b"/>
+    <s v="$-1$"/>
+    <s v="$0$"/>
+    <s v="$1$"/>
+    <s v="$2$"/>
+    <s v="$3$"/>
+    <s v="วิธีทำ: (โจทย์ซ้ำกับข้อ 17) จาก $f'(1)=3$ จะได้ $a+b=3 \Rightarrow b=3-a$ อินทิเกรตหา $f(x)$ แล้วใช้ $f(0)=1$ ได้ค่าคงที่ $C=1$ แทน $f(1)=2$ แล้วแก้สมการจะได้ $a=3, b=0$ จะได้ $f(x) = x^3+1$ ดังนั้น $f(-1) = (-1)^3+1 = 0$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดเกิดจากการอินทิเกรตผิดสูตร หรือแก้สมการสองตัวแปรหาค่า a, b ผิดพลาด"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <n v="0.6"/>
+    <n v="0.45"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="57"/>
+    <s v="ถ้าพื้นที่ที่ปิดล้อมด้วยเส้นโค้ง $y = x^2 - 4x + 3$ และแกน $X$ มีค่าเท่ากับ $A$ และพื้นที่ที่ปิดล้อมด้วย $y = -x^2 + 4x - 3$ และแกน $X$ มีค่าเท่ากับ $B$ จงหา $A + B$"/>
+    <s v="c"/>
+    <s v="$2$"/>
+    <s v=" $\\frac{4}{3}$"/>
+    <s v=" $\\frac{8}{3}$"/>
+    <s v="$4$"/>
+    <s v=" $\\frac{16}{3}$"/>
+    <s v="วิธีทำ: ทั้งสองฟังก์ชันเป็นพาราโบลาที่หน้าตาเหมือนกันแค่คว่ำกับหงาย จุดตัดแกน $X$ คือ $x=1, 3$ พื้นที่ $A = \left| \int_{1}^{3} (x^2-4x+3) dx \right| = \left| [\frac{x^3}{3} - 2x^2 + 3x]_{1}^{3} \right| = \frac{4}{3}$ เนื่องจากสมมาตรกัน พื้นที่ $B$ ก็เท่ากับ $4/3$ ด้วย ดังนั้น $A+B = \frac{8}{3}$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ D และ E เกิดจากการอินทิเกรตเลขผิด ช้อยส์ B ($4/3$) คือหาพื้นที่แค่ส่วนเดียวแล้วลืมนำมาบวกกัน"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="0.75"/>
+    <n v="0.55000000000000004"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="58"/>
+    <s v="จงหาค่าของ $\int_{0}^{3} (x + 1)\sqrt{x + 1} dx$"/>
+    <s v="c"/>
+    <s v=" $\\frac{54}{5}$"/>
+    <s v="$\\frac{58}{5}$"/>
+    <s v="$\\frac{62}{5}$"/>
+    <s v=" $\\frac{64}{5}$"/>
+    <s v="$\\frac{70}{5}$"/>
+    <s v="วิธีทำ: รวบเลขชี้กำลังจะได้ $\int_{0}^{3} (x+1)^{3/2} dx$ ใช้วิธีเปลี่ยนตัวแปร $u = x+1, du = dx$ จะได้ $\int_{1}^{4} u^{3/2} du = [\frac{2}{5} u^{5/2}]_{1}^{4} = \frac{2}{5} (4^{5/2} - 1^{5/2}) = \frac{2}{5} (32 - 1) = \frac{62}{5}$ วิเคราะห์ช้อยส์หลอก: ช้อยส์อื่น ๆ ล้วนเกิดจากการคิดเลขเศษส่วนและเลขยกกำลังผิดพลาดในขั้นตอนสุดท้ายของการแทนค่าขอบเขต"/>
+    <x v="1"/>
+    <x v="8"/>
+    <x v="18"/>
+    <x v="1"/>
+    <n v="0.7"/>
+    <n v="0.6"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="59"/>
+    <s v="จงหาค่าของ $\int (3x^2 - 2x + 5) dx$"/>
+    <s v="a"/>
+    <s v="$x^3 - x^2 + 5x + C$"/>
+    <s v=" $3x^3 - 2x^2 + 5x + C$"/>
+    <s v="$x^3 - x^2 + 5 + C$"/>
+    <s v="$x^3 - x^2 + 5x$"/>
+    <s v="$x^3 - x^2 + 5x + 1$"/>
+    <s v="วิธีทำ: (โจทย์ซ้ำกับข้อ 2) ใช้อินทิเกรตพหุนาม (Power Rule) จะได้ $\frac{3x^3}{3} - \frac{2x^2}{2} + 5x + C = x^3 - x^2 + 5x + C$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ B อินทิเกรตผิดสูตร ช้อยส์ C ลืมอินทิเกรตค่าคงที่ ช้อยส์ D และ E ขาดความเข้าใจเรื่องปริพันธ์ไม่จำกัดเขตโดยลืมบวกค่าคงที่ $C$"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="3"/>
+    <n v="0.2"/>
+    <n v="0.3"/>
+    <s v="correct_answer"/>
+    <s v="wrong_integration_formula"/>
+    <s v="constant_derivative_error"/>
+    <s v="forgot_plus_c"/>
+    <s v="forgot_plus_c"/>
+  </r>
+  <r>
+    <n v="60"/>
+    <s v="กำหนดให้ $f^{\prime\prime}(x) = 12x$ จงหา $f(x)$ เมื่อ $f^{\prime}(0) = 1$ และ $f(0) = 2$"/>
+    <s v="a"/>
+    <s v="$2x^3 + x + 2$"/>
+    <s v="$2x^3 + x$"/>
+    <s v="$4x^3 + x + 2$"/>
+    <s v="$2x^2 + x + 2$"/>
+    <s v="$2x^3 + 2$"/>
+    <s v="วิธีทำ: อินทิเกรต $f''(x)$ จะได้ $f'(x) = 6x^2 + C_1$ จาก $f'(0) = 1$ จะได้ $C_1 = 1$ ดังนั้น $f'(x) = 6x^2 + 1$ อินทิเกรตอีกครั้งจะได้ $f(x) = 2x^3 + x + C_2$ จาก $f(0) = 2$ จะได้ $C_2 = 2$ ดังนั้น $f(x) = 2x^3 + x + 2$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดเกิดจากการลืมบวกค่าคงที่ $C$ ในขั้นตอนการอินทิเกรต หรืออินทิเกรตผิดสูตรเช่นนำสัมประสิทธิ์ไปหารเลขชี้กำลังเดิม"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <n v="0.4"/>
+    <n v="0.4"/>
+    <s v="correct_answer"/>
+    <s v="forgot_plus_c"/>
+    <s v="wrong_integration_formula"/>
+    <s v="wrong_integration_formula"/>
+    <s v="forgot_plus_c"/>
+  </r>
+  <r>
+    <n v="61"/>
+    <s v="จงหาพื้นที่ที่ปิดล้อมด้วยเส้นโค้ง $y = x^2$ และ $y = x$"/>
+    <s v="b"/>
+    <s v="$\\frac{1}{12}$"/>
+    <s v="$\\frac{1}{6}$"/>
+    <s v=" $\\frac{1}{3}$"/>
+    <s v=" $\\frac{1}{2}$"/>
+    <s v="$1$"/>
+    <s v="วิธีทำ: หาจุดตัดโดยตั้ง $x^2 = x \Rightarrow x(x-1) = 0$ ได้ $x = 0, 1$ ในช่วงนี้เส้นตรง $y=x$ อยู่เหนือพาราโบลา ตั้งสมการพื้นที่ $\int_{0}^{1} (x - x^2) dx = [\frac{x^2}{2} - \frac{x^3}{3}]_{0}^{1} = \frac{1}{2} - \frac{1}{3} = \frac{1}{6}$ วิเคราะห์ช้อยส์หลอก: ช้อยส์อื่นๆ เกิดจากการลบเศษส่วนผิดพลาด หรือสลับตำแหน่งเอา $x^2$ ตั้งลบด้วย $x$ แล้วลืมใส่ค่าสัมบูรณ์"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="1"/>
+    <n v="0.5"/>
+    <n v="0.45"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="62"/>
+    <s v="ถ้า $f(x)$ ต่อเนื่องบน $[a, b]$ และ $\displaystyle \int_a^b f(x) dx = 10$ จงหาค่าของ $\displaystyle \int_a^b 2f(x) dx$"/>
+    <s v="c"/>
+    <s v=" $5$"/>
+    <s v=" $10$"/>
+    <s v=" $20$"/>
+    <s v=" $40$"/>
+    <s v="หาค่าไม่ได้"/>
+    <s v="วิธีทำ: จากสมบัติของอินทิกรัลจำกัดเขต สามารถดึงค่าคงที่ออกมานอกเครื่องหมายอินทิเกรตได้ $\int_{a}^{b} 2f(x) dx = 2 \int_{a}^{b} f(x) dx = 2(10) = 20$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดเกิดจากความไม่เข้าใจสมบัติของอินทิกรัล เช่นนำไปหารสอง ไม่นำไปคูณ หรือนำค่ายกกำลัง"/>
+    <x v="1"/>
+    <x v="8"/>
+    <x v="9"/>
+    <x v="3"/>
+    <n v="0.35"/>
+    <n v="0.4"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+  </r>
+  <r>
+    <n v="63"/>
+    <s v="ให้ $f$ เป็นฟังก์ชันหนึ่งต่อหนึ่ง โดย $f^{-1}(x) = \frac{2x}{x+1}$ พิจารณาข้อความ (ก) $2f^{\prime}(4) - f(4) = 3$, (ข) $f^{\prime\prime}(f(4)) = f^{\prime\prime}(f^{\prime}(4))$, (ค) $f$ เป็นฟังก์ชันเพิ่มบนช่วง $(0, 2)$"/>
+    <s v="a"/>
+    <s v="(ก) และ (ข) ถูก แต่ (ค) ผิด"/>
+    <s v="(ก) และ (ค) ถูก แต่ (ข) ผิด"/>
+    <s v="(ข) และ (ค) ถูก แต่ (ก) ผิด "/>
+    <s v="ถูกทั้งสามข้อ"/>
+    <s v="ผิดทั้งสามข้อ"/>
+    <s v="วิธีทำ: หา $f(x)$ โดยสลับตัวแปร จะได้ $f(x) = \frac{x}{2-x}$ หาอนุพันธ์ $f'(x) = \frac{2}{(2-x)^2}$ จะพบว่า $f'(x) &gt; 0$ เสมอเมื่อ $x \ne 2$ ดังนั้น (ค) ถูกต้อง ส่วน $f(4) = -2$ และ $f'(4) = 1/2$ ทำให้ (ก) $2(1/2) - (-2) = 3$ ถูกต้อง สำหรับ (ข) เมื่อคำนวณจะได้ $f''(-2) \ne f''(1/2)$ จึงผิด (หมายเหตุ: ช้อยส์ถูกตัดทอนแต่อิงจากเฉลย A คือข้อที่ระบุว่า ก และ ค ถูก) วิเคราะห์ช้อยส์หลอก: เนื่องจากช้อยส์ปลายทางถูกตัดทอน จึงระบุเป็น Error Code ที่เกี่ยวข้องกับการประเมินข้อความผิด"/>
+    <x v="0"/>
+    <x v="10"/>
+    <x v="19"/>
+    <x v="0"/>
+    <n v="0.8"/>
+    <n v="0.65"/>
+    <s v="correct_answer"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+  </r>
+  <r>
+    <n v="64"/>
+    <s v="กำหนดให้ $P(x)$ เป็นพหุนามดีกรี $2567$ ที่มีสัมประสิทธิ์เป็นจำนวนจริง ให้ $x_1, \dots, x_k$ เป็นรากจริงที่แตกต่างกันของ $P(x)$ และ $n_i$ คือจำนวนน้อยสุดที่ทำให้ $P^{(n_i)}(x_i) \ne 0$"/>
+    <s v="b"/>
+    <s v="$2566$"/>
+    <s v="$2567$"/>
+    <s v="$k$"/>
+    <s v="$2k$"/>
+    <s v="หาค่าไม่ได้"/>
+    <s v="วิธีทำ: (โจทย์ถูกตัดทอนแต่คาดว่าถามถึงผลรวมของ $n_i$) ค่า $n_i$ ในที่นี้คือ Multiplicity หรือจำนวนความซ้ำของราก $x_i$ ตามทฤษฎีบทพีชคณิต พหุนามดีกรี $n$ จะมีผลรวมของความซ้ำของราก (ทั้งจริงและเชิงซ้อน) สูงสุดเท่ากับ $n$ ดังนั้นผลรวมสูงสุดที่เป็นไปได้คือดีกรีของพหุนาม ซึ่งก็คือ $2567$ วิเคราะห์ช้อยส์หลอก: ช้อยส์อื่นเป็นการหลอกด้วยตัวเลขใกล้เคียง หรือขาดความเข้าใจในทฤษฎีบทพื้นฐานของพีชคณิต"/>
+    <x v="0"/>
+    <x v="11"/>
+    <x v="20"/>
+    <x v="0"/>
+    <n v="0.75"/>
+    <n v="0.6"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="correct_answer"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="conceptual_misunderstanding"/>
+  </r>
+  <r>
+    <n v="65"/>
+    <s v="กำหนดให้ $f(x) = x^3 + 2x - 1$ จงหาค่าของ $(f^{-1})^{\prime}(2)$"/>
+    <s v="b"/>
+    <s v="$1/4$"/>
+    <s v="$1/5$"/>
+    <s v="$1/8$"/>
+    <s v="$5$"/>
+    <s v="$4$"/>
+    <s v="วิธีทำ: ใช้สูตรอนุพันธ์ฟังก์ชันผกผัน $(f^{-1})'(y) = \frac{1}{f'(x)}$ ขั้นแรกหา $x$ ที่ทำให้ $f(x) = 2 \Rightarrow x^3 + 2x - 1 = 2 \Rightarrow x^3 + 2x - 3 = 0$ จะได้ $x=1$ ถัดมาหา $f'(x) = 3x^2 + 2$ ดังนั้น $f'(1) = 5$ นำไปแทนในสูตรจะได้ $\frac{1}{5}$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดเกิดจากการแก้สมการหาค่า $x$ ผิด หรือลืมส่วนกลับ (ตอบ $5$ ทันที)"/>
+    <x v="0"/>
+    <x v="10"/>
+    <x v="9"/>
+    <x v="0"/>
+    <n v="0.85"/>
+    <n v="0.7"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="66"/>
+    <s v="กำหนดให้ $g(x)$ หาอนุพันธ์ได้ โดยที่ $g(1) = 3$ และ $g^{\prime}(1) = 5$ ถ้า $h(x) = g(x^2)(x^2 + 1)$ จงหาค่าของ $h^{\prime}(1)$"/>
+    <s v="c"/>
+    <s v="$10$"/>
+    <s v="$14$"/>
+    <s v="$16$"/>
+    <s v="$20$"/>
+    <s v="$26$"/>
+    <s v="วิธีทำ: (หมายเหตุ: คำตอบทางคณิตศาสตร์คือ $26$ ซึ่งตรงกับช้อยส์ E แต่เฉลยในตารางระบุ C=$16$) หาอนุพันธ์ด้วยกฎผลคูณและกฎลูกโซ่ $h'(x) = g'(x^2)(2x)(x^2+1) + g(x^2)(2x)$ แทนค่า $x=1$ จะได้ $h'(1) = g'(1)(2)(2) + g(1)(2) = 5(4) + 3(2) = 26$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ C (เฉลย) และช้อยส์อื่นๆ เกิดจากการลืมคูณอนุพันธ์ไส้ (กฎลูกโซ่) หรือใช้กฎผลคูณผิดพลาดในขั้นตอนใดขั้นตอนหนึ่ง"/>
+    <x v="0"/>
+    <x v="12"/>
+    <x v="0"/>
+    <x v="1"/>
+    <n v="0.7"/>
+    <n v="0.55000000000000004"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="67"/>
+    <s v="จงหาอนุพันธ์อันดับที่ 2 ของ $f(x) = \ln(2x + 1)$ ที่ $x = 0.5$"/>
+    <s v="b"/>
+    <s v=" $-1/2$"/>
+    <s v=" $-1$"/>
+    <s v=" $-2$"/>
+    <s v=" $1$"/>
+    <s v=" $-1/4$"/>
+    <s v="วิธีทำ: หาอนุพันธ์อันดับหนึ่ง $f'(x) = \frac{1}{2x+1} \cdot 2 = 2(2x+1)^{-1}$ หาอนุพันธ์อันดับสอง $f''(x) = -2(2x+1)^{-2} \cdot 2 = \frac{-4}{(2x+1)^2}$ แทนค่า $x = 0.5$ จะได้ $f''(0.5) = \frac{-4}{(2(0.5)+1)^2} = \frac{-4}{2^2} = -1$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ผิดเกิดจากการลืมดิฟไส้ (กฎลูกโซ่) ในอนุพันธ์อันดับหนึ่งหรือสอง หรือคิดเลขเศษส่วนพลาด"/>
+    <x v="0"/>
+    <x v="13"/>
+    <x v="21"/>
+    <x v="1"/>
+    <n v="0.65"/>
+    <n v="0.55000000000000004"/>
+    <s v="forgot_chain_rule_inner"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="sign_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="68"/>
+    <s v="กำหนดให้ $f(x)$ เป็นพหุนาม ถ้า $f(\sqrt{x} - 1) = x$ เมื่อ $x &gt; 0$ แล้ว $f^{\prime}(1)$ เท่ากับเท่าใด"/>
+    <s v="c"/>
+    <s v=" $1$"/>
+    <s v=" $2$"/>
+    <s v=" $4$"/>
+    <s v=" $5$"/>
+    <s v=" $8$"/>
+    <s v="วิธีทำ: (โจทย์ซ้ำกับข้อ 4) หาอนุพันธ์ทั้งสองข้างด้วยกฎลูกโซ่ $f'(\sqrt{x}-1) \cdot \frac{1}{2\sqrt{x}} = 1$ เมื่อต้องการหา $f'(1)$ ต้องตั้ง $\sqrt{x}-1 = 1 \Rightarrow x=4$ นำไปแทนค่าได้ $f'(1) \cdot \frac{1}{4} = 1 \Rightarrow f'(1) = 4$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ผิดเกิดจากการแทนค่า $x=1$ ลงไปดื้อๆ หรือประเมินฟังก์ชันประกอบผิด"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="0.8"/>
+    <n v="0.6"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="composite_evaluation_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="69"/>
+    <s v="กำหนดให้ $f$ เป็นฟังก์ชัน โดยที่ $f^{\prime}(x) = 2x + 1$ ถ้า $h(x) = f(x^2)$ แล้ว $h^{\prime}(x)$ มีค่าเท่ากับเท่าใด"/>
+    <s v="d"/>
+    <s v="$4x + 2$"/>
+    <s v="$2x^2 + 1$"/>
+    <s v="$4x^2 + 2x$"/>
+    <s v="$4x^3 + 2x$"/>
+    <s v="$4x^3 + 4x$"/>
+    <s v="วิธีทำ: หาอนุพันธ์ด้วยกฎลูกโซ่ $h'(x) = f'(x^2) \cdot \frac{d}{dx}(x^2) = f'(x^2) \cdot 2x$ จากที่โจทย์กำหนด $f'(x) = 2x+1$ เมื่อแทน $x$ ด้วย $x^2$ จะได้ $f'(x^2) = 2x^2+1$ นำกลับไปแทนในสมการแรกจะได้ $h'(x) = (2x^2+1)(2x) = 4x^3 + 2x$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดเกิดจากการลืมคูณดิฟไส้ $2x$ หรือสับสนนำ $f'(x)$ ไปยกกำลังสองแทนการแทนค่า"/>
+    <x v="0"/>
+    <x v="14"/>
+    <x v="17"/>
+    <x v="1"/>
+    <n v="0.45"/>
+    <n v="0.4"/>
+    <s v="forgot_chain_rule_inner"/>
+    <s v="forgot_chain_rule_inner"/>
+    <s v="composite_evaluation_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="70"/>
+    <s v="กำหนดให้ $f(x) = \left|x^2 - 9\right|$ พิจารณาข้อความ (ก) $f^{\prime}(3)$ หาค่าได้ (ข) $f^{\prime}(-3)$ หาค่าไม่ได้ (ค) $f^{\prime}(0) = 0$ ข้อใดถูกต้อง"/>
+    <s v="d"/>
+    <s v="(ก) เท่านั้น"/>
+    <s v=" (ข) เท่านั้น "/>
+    <s v=" (ค) เท่านั้น "/>
+    <s v=" (ข) และ (ค) ถูก"/>
+    <s v="ถูกทุกข้อ"/>
+    <s v="วิธีทำ: ฟังก์ชันค่าสัมบูรณ์จะมีจุดหักมุม (Cusp) ที่ทำให้ค่าในค่าสัมบูรณ์เป็นศูนย์ ซึ่งคือ $x = 3, -3$ ที่จุดเหล่านี้ฟังก์ชันจะหาอนุพันธ์ไม่ได้ ดังนั้น (ก) ผิด และ (ข) ถูก สำหรับ $x=0$ ค่าในสัมบูรณ์ติดลบ จึงถอดได้ $f(x) = 9-x^2$ ซึ่ง $f'(x) = -2x \Rightarrow f'(0) = 0$ ดังนั้น (ค) ถูกต้อง วิเคราะห์ช้อยส์หลอก: ช้อยส์อื่นเกิดจากความไม่เข้าใจนิยามความต่อเนื่องและการหาอนุพันธ์ของฟังก์ชันค่าสัมบูรณ์"/>
+    <x v="0"/>
+    <x v="9"/>
+    <x v="22"/>
+    <x v="0"/>
+    <n v="0.75"/>
+    <n v="0.6"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="correct_answer"/>
+    <s v="conceptual_misunderstanding"/>
+  </r>
+  <r>
+    <n v="71"/>
+    <s v="กำหนดให้ $f^{\prime}(x) = 2x + 1$ และ $h(x) = f(x^2)$ แล้ว $h^{\prime}(x)$ มีค่าเท่ากับเท่าใด"/>
+    <s v="d"/>
+    <s v="$4x + 2$"/>
+    <s v="$2x^2 + 1$"/>
+    <s v="$4x^2 + 2x$"/>
+    <s v="$4x^3 + 2x$"/>
+    <s v="$4x^3 + 4x$"/>
+    <s v="วิธีทำ: (โจทย์ซ้ำกับข้อ 70 ทุกประการ) $h'(x) = f'(x^2) \cdot 2x = (2x^2+1)(2x) = 4x^3 + 2x$ วิเคราะห์ช้อยส์หลอก: ข้อผิดพลาดเกิดจากการลืมดิฟไส้หรือประเมินฟังก์ชันประกอบผิด"/>
+    <x v="0"/>
+    <x v="14"/>
+    <x v="17"/>
+    <x v="1"/>
+    <n v="0.45"/>
+    <n v="0.4"/>
+    <s v="forgot_chain_rule_inner"/>
+    <s v="forgot_chain_rule_inner"/>
+    <s v="composite_evaluation_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="72"/>
+    <s v="กำหนดให้ $f(x) = x^3 - 3x^2 + 4$ จงหา $(f^{-1})^{\prime}(4)$"/>
+    <s v="a"/>
+    <s v="$1/9$"/>
+    <s v="$1/3$"/>
+    <s v="$3$"/>
+    <s v="$9$"/>
+    <s v="$-1/9$"/>
+    <s v="วิธีทำ: ใช้สูตร $(f^{-1})'(y) = \frac{1}{f'(x)}$ เริ่มจากหา $x$ ที่ทำให้ $x^3 - 3x^2 + 4 = 4 \Rightarrow x^2(x-3) = 0$ โดยทั่วไปโจทย์อนุพันธ์ผกผันจะพิจารณาช่วงที่ฟังก์ชันเป็น 1-1 ซึ่งราก $x=3$ จะใช้งานได้ ($x=0$ เป็นจุดวิกฤต) หา $f'(x) = 3x^2 - 6x$ แทน $x=3$ จะได้ $f'(3) = 27 - 18 = 9$ นำไปกลับเศษส่วนจะได้ $\frac{1}{9}$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดเกิดจากการตอบ $f'(3)$ ตรงๆ โดยลืมกลับเศษส่วน หรือคิดเลขผิด"/>
+    <x v="0"/>
+    <x v="10"/>
+    <x v="9"/>
+    <x v="0"/>
+    <n v="0.8"/>
+    <n v="0.65"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+    <s v="sign_error"/>
+  </r>
+  <r>
+    <n v="73"/>
+    <s v="กำหนดให้ $f(x) = \begin{cases} \frac{x^2-4}{x-2}, &amp; x \ne 2 \\ a, &amp; x = 2 \end{cases}$ และ $g(x) = \begin{cases} \frac{x^2-1}{x-1}, &amp; x \ne 1 \\ b, &amp; x = 1 \end{cases}$ ถ้า $f, g$ ต่อเนื่องทุกจุด แล้ว $f(a+b)$ เท่ากับเท่าใด"/>
+    <s v="c"/>
+    <s v="$4$ "/>
+    <s v=" $6$ "/>
+    <s v="$8$"/>
+    <s v="$9$ "/>
+    <s v="$16$"/>
+    <s v="วิธีทำ: ความต่อเนื่องแปลว่าลิมิตเท่ากับค่าฟังก์ชัน $a = \lim_{x \to 2} \frac{(x-2)(x+2)}{x-2} = 4$ และ $b = \lim_{x \to 1} \frac{(x-1)(x+1)}{x-1} = 2$ ต้องการหา $f(a+b) = f(4+2) = f(6)$ ซึ่ง $6 \ne 2$ จึงใช้เงื่อนไขบน $f(6) = \frac{36-4}{6-2} = \frac{32}{4} = 8$ (หรือแทนในฟังก์ชันที่ตัดทอนแล้ว $x+2 = 6+2 = 8$) วิเคราะห์ช้อยส์หลอก: ช้อยส์อื่นเกิดจากการหาค่าลิมิตผิดพลาด หรือบวกเลข a, b พลาด"/>
+    <x v="2"/>
+    <x v="6"/>
+    <x v="9"/>
+    <x v="0"/>
+    <n v="0.75"/>
+    <n v="0.6"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="74"/>
+    <s v="กำหนดให้ $f(x) = \begin{cases} \frac{\sqrt{x}-2}{x-4}, &amp; x &gt; 4 \\ ax+b, &amp; 0 &lt; x \le 4 \\ x^2+4x, &amp; x \le 0 \end{cases}$ ถ้า $f$ ต่อเนื่องทุกจุด แล้ว $f(a+b)$ เท่ากับเท่าใด"/>
+    <s v="c"/>
+    <s v="$-8$ "/>
+    <s v="$-6$ "/>
+    <s v="$-4$ "/>
+    <s v="$0$ "/>
+    <s v="$4$ "/>
+    <s v="วิธีทำ: (หมายเหตุ: มีความเป็นไปได้สูงที่โจทย์ตั้งค่าตัวแปรผิดพลาด) ความต่อเนื่องที่ $x=0$ ทำให้ $b = 0^2+4(0) = 0$ ความต่อเนื่องที่ $x=4$ คือ $\lim_{x \to 4} \frac{1}{\sqrt{x}+2} = \frac{1}{4}$ ทำให้ $4a = 1/4 \Rightarrow a=1/16$ ซึ่งโจทย์ถาม $f(a+b) = f(1/16) = \frac{1}{256}$ แต่เฉลยคือ C ($-4$) คาดว่าโจทย์จริงตั้งใจให้สมการหรือตัวเลขต่างออกไปเพื่อให้ได้ $a, b$ ที่ลงตัวกว่านี้ วิเคราะห์ช้อยส์หลอก: ระบุเป็น Unclassified Error เนื่องจากโจทย์น่าจะมีความคลาดเคลื่อนในตัวเลข"/>
+    <x v="2"/>
+    <x v="6"/>
+    <x v="9"/>
+    <x v="0"/>
+    <n v="0.8"/>
+    <n v="0.65"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+    <s v="correct_answer"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+  </r>
+  <r>
+    <n v="75"/>
+    <s v="กำหนดให้ $f(x) = \begin{cases} \frac{x^2+2x-3}{x-1}, &amp; x &gt; 1 \\ x^2+ax+b, &amp; x \le 1 \end{cases}$ ถ้า $f$ ต่อเนื่องที่ $x=1$ และ $f^{\prime}(0)=4$ แล้ว $a+b$ เท่ากับเท่าใด"/>
+    <s v="c"/>
+    <s v="$1$ "/>
+    <s v="$2$ "/>
+    <s v="$3$ "/>
+    <s v="$4$ "/>
+    <s v="$5$ "/>
+    <s v="วิธีทำ: จาก $f'(0)=4$ จะใช้ฟังก์ชันช่วงล่าง ได้ $f'(x) = 2x+a \Rightarrow f'(0) = a = 4$ ความต่อเนื่องที่ $x=1$ ลิมิตขวาคือ $\lim_{x \to 1^+} \frac{(x-1)(x+3)}{x-1} = 4$ ลิมิตซ้ายคือ $1^2 + 4(1) + b = 5+b$ จับเท่ากัน $5+b = 4 \Rightarrow b=-1$ ดังนั้น $a+b = 4 + (-1) = 3$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดเกิดจากการแยกตัวประกอบลิมิตผิด เครื่องหมายผิดตอนแก้สมการ หรือดิฟฟังก์ชันผิด"/>
+    <x v="2"/>
+    <x v="6"/>
+    <x v="23"/>
+    <x v="0"/>
+    <n v="0.75"/>
+    <n v="0.6"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="76"/>
+    <s v="กำหนดให้ $f(x) = \begin{cases} x+\sqrt{x^2+5}, &amp; x \ge a \\ \frac{15}{\sqrt{x^2+5}}, &amp; x &lt; a \end{cases}$ ถ้า $f$ ต่อเนื่องทุกจำนวนจริง แล้ว $a^2+a$ เท่ากับเท่าใด"/>
+    <s v="c"/>
+    <s v="$2$ "/>
+    <s v="$4$ "/>
+    <s v="$6$ "/>
+    <s v="$8$ "/>
+    <s v="$12$ "/>
+    <s v="วิธีทำ: ความต่อเนื่องที่ $x=a$ คือ $a+\sqrt{a^2+5} = \frac{15}{\sqrt{a^2+5}}$ คูณไขว้จะได้ $a\sqrt{a^2+5} + a^2 + 5 = 15 \Rightarrow a\sqrt{a^2+5} = 10-a^2$ ยกกำลังสองทั้งสองข้าง $a^2(a^2+5) = 100 - 20a^2 + a^4$ แก้สมการได้ $a^2 = 4 \Rightarrow a=\pm2$ ตรวจคำตอบพบว่ามีเพียง $a=2$ ที่ทำให้สมการก่อนยกกำลังสองเป็นจริง ดังนั้น $a^2+a = 4+2 = 6$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ผิดเกิดจากการไม่ได้ตรวจคำตอบและนำรากแปลกปลอม $a=-2$ ไปคำนวณ หรือแก้สมการยกกำลังสองผิดพลาด"/>
+    <x v="2"/>
+    <x v="6"/>
+    <x v="4"/>
+    <x v="0"/>
+    <n v="0.8"/>
+    <n v="0.6"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="77"/>
+    <s v="กำหนดให้ $f$ เป็นฟังก์ชันที่หาอนุพันธ์ได้ และ $g(x) = (f(x))^2$ ถ้า $f(7)=3$ และ $g^{\prime}(7)=1$ แล้วอนุพันธ์ของ $f(2x^2+4x-9)$ ที่ $x=2$ มีค่าเท่าใด"/>
+    <s v="b"/>
+    <s v="$1$ "/>
+    <s v="$2$ "/>
+    <s v="$3$ "/>
+    <s v="$4$ "/>
+    <s v="$6$ "/>
+    <s v="วิธีทำ: (โจทย์ซ้ำกับข้อ 1) กฎลูกโซ่ $g'(x) = 2f(x)f'(x) \Rightarrow 1 = 2(3)f'(7) \Rightarrow f'(7) = 1/6$ จากนั้นให้ $h(x) = f(2x^2+4x-9)$ จะได้ $h'(x) = f'(2x^2+4x-9) \cdot (4x+4)$ แทน $x=2$ จะได้ $h'(2) = f'(7) \cdot 12 = (1/6) \cdot 12 = 2$ วิเคราะห์ช้อยส์หลอก: เกิดจากคิดเลขผิด หรือไม่เข้าใจการประยุกต์กฎลูกโซ่ซ้อนกัน"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
+    <n v="0.6"/>
+    <n v="0.55000000000000004"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+  <r>
+    <n v="78"/>
+    <s v="กำหนดให้ $P(x) = (x^{10^0} + x^{10^1} + x^{10^2} + \dots + x^{10^9})^9$ ให้ $A$ เป็นจำนวนหลักของ $P^{\prime}(1)$ และ $B$ เป็นผลบวกเลขโดดของ $P^{\prime}(1)$ จงหา $A+B$"/>
+    <s v="c"/>
+    <s v="$19$ "/>
+    <s v="$23$ "/>
+    <s v="$28$ "/>
+    <s v="$32$ "/>
+    <s v="$36$ "/>
+    <s v="วิธีทำ: (หมายเหตุ: คำตอบทางคณิตศาสตร์คือ $108$ แต่เฉลยคือ C=$28$) ให้ $Q(x) = x^{1} + x^{10} + \dots + x^{10^9}$ จะได้ $Q(1) = 10$ หา $Q'(x) = 1 + 10x^9 + \dots$ จะได้ $Q'(1) = 1 + 10 + \dots + 10^9 = 1,111,111,111$ หา $P'(x) = 9(Q(x))^8 \cdot Q'(x)$ แทนค่าได้ $P'(1) = 9(10^8)(1111111111) = 9999999999 \times 10^8$ ซึ่งมีจำนวนหลัก $A=18$ และผลบวกเลขโดด $B=90$ ได้ $A+B=108$ คาดว่าโจทย์มีความผิดพลาดในเลขชี้กำลังหรือตัวเลือกเฉลย วิเคราะห์ช้อยส์หลอก: ช้อยส์ในโจทย์มีค่าต่ำเกินกว่าความเป็นจริงทางคณิตศาสตร์ จึงจัดเป็น Unclassified Error"/>
+    <x v="0"/>
+    <x v="14"/>
+    <x v="20"/>
+    <x v="1"/>
+    <n v="0.7"/>
+    <n v="0.6"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+    <s v="correct_answer"/>
+    <s v="unclassified_error"/>
+    <s v="unclassified_error"/>
+  </r>
+  <r>
+    <n v="79"/>
+    <s v="กำหนดให้ $f(x) = x^3 + 2x + 3$ และ $g(x) = f^{-1}(x)$ แล้ว $g^{\prime}(6)$ เท่ากับข้อใด"/>
+    <s v="c"/>
+    <s v="$1/2$ "/>
+    <s v=" $1/3$ "/>
+    <s v=" $1/5$ "/>
+    <s v="$1/14$ "/>
+    <s v="$5$"/>
+    <s v="วิธีทำ: หา $x$ ที่ $f(x)=6 \Rightarrow x^3+2x+3=6 \Rightarrow x^3+2x-3=0 \Rightarrow x=1$ จากกฎฟังก์ชันผกผัน $g'(6) = \frac{1}{f'(1)}$ หาอนุพันธ์ $f'(x) = 3x^2+2 \Rightarrow f'(1) = 3(1)+2 = 5$ ดังนั้น $g'(6) = \frac{1}{5}$ วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ผิดเกิดจากการตอบ $f'(1)$ โดยไม่กลับเศษส่วน หรือแก้สมการพหุนามหาค่า $x$ พลาด"/>
+    <x v="0"/>
+    <x v="10"/>
+    <x v="9"/>
+    <x v="0"/>
+    <n v="0.85"/>
+    <n v="0.65"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="conceptual_misunderstanding"/>
+  </r>
+  <r>
+    <n v="80"/>
+    <s v="กำหนดให้ $f(x) = \begin{cases} (x+1)^2-5, &amp; x &lt; -1 \\ x-1, &amp; -1 \le x \le 1 \\ (x-1)^2-5, &amp; x &gt; 1 \end{cases}$ แล้ว $(f \circ f)^{\prime}(2)$ เท่ากับข้อใด"/>
+    <s v="b"/>
+    <s v="$12$ "/>
+    <s v="$8 "/>
+    <s v="$0$ "/>
+    <s v="$-8$ "/>
+    <s v="$-12$ "/>
+    <s v="วิธีทำ: (หมายเหตุ: คำตอบทางคณิตศาสตร์คือ $-12$ แต่เฉลยคือ B=$8$) หา $f(2)$ จากกรณีล่างสุด $(2-1)^2-5 = -4$ จากกฎลูกโซ่ $(f \circ f)'(2) = f'(f(2)) \cdot f'(2) = f'(-4) \cdot f'(2)$ หา $f'(2)$ จากอนุพันธ์ล่าง $2(x-1) \Rightarrow 2$ หา $f'(-4)$ จากอนุพันธ์บน $2(x+1) \Rightarrow 2(-3) = -6$ นำมาคูณกันได้ $(-6)(2) = -12$ ตัวเฉลยอาจมาจากความผิดพลาดของการพิมพ์โจทย์ต้นฉบับ วิเคราะห์ช้อยส์หลอก: ช้อยส์ที่ถูกต้องตามคณิตศาสตร์คือ E ($-12$) ช้อยส์อื่นๆ รวมถึงเฉลยเกิดจากการแทนค่าเงื่อนไขผิดช่วงหรือคิดเลขผิด"/>
+    <x v="0"/>
+    <x v="14"/>
+    <x v="17"/>
+    <x v="0"/>
+    <n v="0.85"/>
+    <n v="0.65"/>
+    <s v="arithmetic_error"/>
+    <s v="correct_answer"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+    <s v="arithmetic_error"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{34BAD308-3109-49BF-9FD2-C956A449B32A}" name="PivotTable1" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="A3:D43" firstHeaderRow="1" firstDataRow="1" firstDataCol="3"/>
+  <pivotFields count="20">
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField axis="axisRow" dataField="1" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="4">
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+      </items>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="11"/>
+        <item x="3"/>
+        <item x="14"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="10"/>
+        <item x="5"/>
+        <item x="2"/>
+        <item x="12"/>
+        <item x="13"/>
+      </items>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="24">
+        <item x="4"/>
+        <item x="0"/>
+        <item x="17"/>
+        <item x="10"/>
+        <item x="22"/>
+        <item x="7"/>
+        <item x="23"/>
+        <item x="9"/>
+        <item x="14"/>
+        <item x="21"/>
+        <item x="2"/>
+        <item x="11"/>
+        <item x="6"/>
+        <item x="8"/>
+        <item x="5"/>
+        <item x="16"/>
+        <item x="12"/>
+        <item x="20"/>
+        <item x="1"/>
+        <item x="19"/>
+        <item x="3"/>
+        <item x="13"/>
+        <item x="15"/>
+        <item x="18"/>
+      </items>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+      </items>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
+          <x14:pivotField fillDownLabels="1"/>
+        </ext>
+      </extLst>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="3">
+    <field x="9"/>
+    <field x="10"/>
+    <field x="11"/>
+  </rowFields>
+  <rowItems count="40">
+    <i>
+      <x/>
+      <x v="2"/>
+      <x v="5"/>
+    </i>
+    <i r="2">
+      <x v="20"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+      <x v="12"/>
+    </i>
+    <i r="1">
+      <x v="11"/>
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="1"/>
+      <x/>
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+      <x v="17"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+      <x v="2"/>
+    </i>
+    <i r="2">
+      <x v="17"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+      <x v="12"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+      <x v="4"/>
+    </i>
+    <i r="2">
+      <x v="16"/>
+    </i>
+    <i r="2">
+      <x v="18"/>
+    </i>
+    <i r="1">
+      <x v="10"/>
+      <x v="7"/>
+    </i>
+    <i r="2">
+      <x v="19"/>
+    </i>
+    <i r="1">
+      <x v="13"/>
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="14"/>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="2"/>
+      <x v="6"/>
+      <x v="2"/>
+    </i>
+    <i r="2">
+      <x v="7"/>
+    </i>
+    <i r="2">
+      <x v="13"/>
+    </i>
+    <i r="2">
+      <x v="15"/>
+    </i>
+    <i r="2">
+      <x v="18"/>
+    </i>
+    <i r="2">
+      <x v="23"/>
+    </i>
+    <i r="1">
+      <x v="9"/>
+      <x/>
+    </i>
+    <i r="2">
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="3"/>
+      <x v="4"/>
+      <x/>
+    </i>
+    <i r="2">
+      <x v="6"/>
+    </i>
+    <i r="2">
+      <x v="7"/>
+    </i>
+    <i r="2">
+      <x v="10"/>
+    </i>
+    <i r="2">
+      <x v="14"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+      <x/>
+    </i>
+    <i r="2">
+      <x v="3"/>
+    </i>
+    <i r="2">
+      <x v="10"/>
+    </i>
+    <i r="2">
+      <x v="11"/>
+    </i>
+    <i r="2">
+      <x v="16"/>
+    </i>
+    <i r="2">
+      <x v="21"/>
+    </i>
+    <i r="2">
+      <x v="22"/>
+    </i>
+    <i r="1">
+      <x v="12"/>
+      <x v="3"/>
+    </i>
+    <i r="2">
+      <x v="8"/>
+    </i>
+    <i r="2">
+      <x v="10"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of main_topic" fld="9" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" fillDownLabelsDefault="1" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2620,32 +4900,1422 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA606220-2C84-495D-811E-C50104B9BB00}">
+  <dimension ref="A3:N43"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
+  <cols>
+    <col min="1" max="1" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:14">
+      <c r="A3" s="22" t="s">
+        <v>345</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>647</v>
+      </c>
+      <c r="F3" t="s">
+        <v>345</v>
+      </c>
+      <c r="G3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" t="s">
+        <v>647</v>
+      </c>
+      <c r="K3" t="s">
+        <v>345</v>
+      </c>
+      <c r="L3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M3" t="s">
+        <v>7</v>
+      </c>
+      <c r="N3" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" t="s">
+        <v>367</v>
+      </c>
+      <c r="B4" t="s">
+        <v>239</v>
+      </c>
+      <c r="C4" t="s">
+        <v>235</v>
+      </c>
+      <c r="D4" s="23">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
+        <v>367</v>
+      </c>
+      <c r="G4" t="s">
+        <v>239</v>
+      </c>
+      <c r="H4" t="s">
+        <v>235</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="K4" t="s">
+        <v>367</v>
+      </c>
+      <c r="L4" t="s">
+        <v>367</v>
+      </c>
+      <c r="M4" t="s">
+        <v>276</v>
+      </c>
+      <c r="N4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" t="s">
+        <v>367</v>
+      </c>
+      <c r="B5" t="s">
+        <v>239</v>
+      </c>
+      <c r="C5" t="s">
+        <v>292</v>
+      </c>
+      <c r="D5" s="23">
+        <v>16</v>
+      </c>
+      <c r="F5" t="s">
+        <v>367</v>
+      </c>
+      <c r="G5" t="s">
+        <v>239</v>
+      </c>
+      <c r="H5" t="s">
+        <v>292</v>
+      </c>
+      <c r="I5">
+        <v>16</v>
+      </c>
+      <c r="L5" t="s">
+        <v>239</v>
+      </c>
+      <c r="M5" t="s">
+        <v>235</v>
+      </c>
+      <c r="N5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" t="s">
+        <v>367</v>
+      </c>
+      <c r="B6" t="s">
+        <v>283</v>
+      </c>
+      <c r="C6" t="s">
+        <v>289</v>
+      </c>
+      <c r="D6" s="23">
+        <v>2</v>
+      </c>
+      <c r="F6" t="s">
+        <v>367</v>
+      </c>
+      <c r="G6" t="s">
+        <v>283</v>
+      </c>
+      <c r="H6" t="s">
+        <v>289</v>
+      </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
+      <c r="M6" t="s">
+        <v>292</v>
+      </c>
+      <c r="N6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" t="s">
+        <v>367</v>
+      </c>
+      <c r="B7" t="s">
+        <v>237</v>
+      </c>
+      <c r="C7" t="s">
+        <v>250</v>
+      </c>
+      <c r="D7" s="23">
+        <v>1</v>
+      </c>
+      <c r="F7" t="s">
+        <v>367</v>
+      </c>
+      <c r="G7" t="s">
+        <v>237</v>
+      </c>
+      <c r="H7" t="s">
+        <v>250</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="L7" t="s">
+        <v>283</v>
+      </c>
+      <c r="M7" t="s">
+        <v>283</v>
+      </c>
+      <c r="N7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" t="s">
+        <v>227</v>
+      </c>
+      <c r="B8" t="s">
+        <v>282</v>
+      </c>
+      <c r="C8" t="s">
+        <v>247</v>
+      </c>
+      <c r="D8" s="23">
+        <v>4</v>
+      </c>
+      <c r="F8" t="s">
+        <v>227</v>
+      </c>
+      <c r="G8" t="s">
+        <v>282</v>
+      </c>
+      <c r="H8" t="s">
+        <v>247</v>
+      </c>
+      <c r="I8">
+        <v>4</v>
+      </c>
+      <c r="M8" t="s">
+        <v>289</v>
+      </c>
+      <c r="N8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" t="s">
+        <v>227</v>
+      </c>
+      <c r="B9" t="s">
+        <v>367</v>
+      </c>
+      <c r="C9" t="s">
+        <v>276</v>
+      </c>
+      <c r="D9" s="23">
+        <v>1</v>
+      </c>
+      <c r="F9" t="s">
+        <v>227</v>
+      </c>
+      <c r="G9" t="s">
+        <v>367</v>
+      </c>
+      <c r="H9" t="s">
+        <v>276</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="L9" t="s">
+        <v>237</v>
+      </c>
+      <c r="M9" t="s">
+        <v>289</v>
+      </c>
+      <c r="N9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" t="s">
+        <v>227</v>
+      </c>
+      <c r="B10" t="s">
+        <v>247</v>
+      </c>
+      <c r="C10" t="s">
+        <v>265</v>
+      </c>
+      <c r="D10" s="23">
+        <v>3</v>
+      </c>
+      <c r="F10" t="s">
+        <v>227</v>
+      </c>
+      <c r="G10" t="s">
+        <v>247</v>
+      </c>
+      <c r="H10" t="s">
+        <v>265</v>
+      </c>
+      <c r="I10">
+        <v>3</v>
+      </c>
+      <c r="M10" t="s">
+        <v>250</v>
+      </c>
+      <c r="N10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" t="s">
+        <v>227</v>
+      </c>
+      <c r="B11" t="s">
+        <v>247</v>
+      </c>
+      <c r="C11" t="s">
+        <v>276</v>
+      </c>
+      <c r="D11" s="23">
+        <v>1</v>
+      </c>
+      <c r="F11" t="s">
+        <v>227</v>
+      </c>
+      <c r="G11" t="s">
+        <v>247</v>
+      </c>
+      <c r="H11" t="s">
+        <v>276</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
+      <c r="K11" t="s">
+        <v>227</v>
+      </c>
+      <c r="L11" t="s">
+        <v>282</v>
+      </c>
+      <c r="M11" t="s">
+        <v>249</v>
+      </c>
+      <c r="N11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" t="s">
+        <v>227</v>
+      </c>
+      <c r="B12" t="s">
+        <v>283</v>
+      </c>
+      <c r="C12" t="s">
+        <v>289</v>
+      </c>
+      <c r="D12" s="23">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>227</v>
+      </c>
+      <c r="G12" t="s">
+        <v>283</v>
+      </c>
+      <c r="H12" t="s">
+        <v>289</v>
+      </c>
+      <c r="I12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
+        <v>246</v>
+      </c>
+      <c r="N12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13" t="s">
+        <v>227</v>
+      </c>
+      <c r="B13" t="s">
+        <v>280</v>
+      </c>
+      <c r="C13" t="s">
+        <v>283</v>
+      </c>
+      <c r="D13" s="23">
+        <v>1</v>
+      </c>
+      <c r="F13" t="s">
+        <v>227</v>
+      </c>
+      <c r="G13" t="s">
+        <v>280</v>
+      </c>
+      <c r="H13" t="s">
+        <v>283</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
+      </c>
+      <c r="L13" t="s">
+        <v>247</v>
+      </c>
+      <c r="M13" t="s">
+        <v>247</v>
+      </c>
+      <c r="N13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" t="s">
+        <v>227</v>
+      </c>
+      <c r="B14" t="s">
+        <v>280</v>
+      </c>
+      <c r="C14" t="s">
+        <v>243</v>
+      </c>
+      <c r="D14" s="23">
+        <v>2</v>
+      </c>
+      <c r="F14" t="s">
+        <v>227</v>
+      </c>
+      <c r="G14" t="s">
+        <v>280</v>
+      </c>
+      <c r="H14" t="s">
+        <v>243</v>
+      </c>
+      <c r="I14">
+        <v>2</v>
+      </c>
+      <c r="L14" t="s">
+        <v>283</v>
+      </c>
+      <c r="M14" t="s">
+        <v>289</v>
+      </c>
+      <c r="N14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15" t="s">
+        <v>227</v>
+      </c>
+      <c r="B15" t="s">
+        <v>280</v>
+      </c>
+      <c r="C15" t="s">
+        <v>250</v>
+      </c>
+      <c r="D15" s="23">
+        <v>1</v>
+      </c>
+      <c r="F15" t="s">
+        <v>227</v>
+      </c>
+      <c r="G15" t="s">
+        <v>280</v>
+      </c>
+      <c r="H15" t="s">
+        <v>250</v>
+      </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
+      <c r="L15" t="s">
+        <v>280</v>
+      </c>
+      <c r="M15" t="s">
+        <v>280</v>
+      </c>
+      <c r="N15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="A16" t="s">
+        <v>227</v>
+      </c>
+      <c r="B16" t="s">
+        <v>266</v>
+      </c>
+      <c r="C16" t="s">
+        <v>285</v>
+      </c>
+      <c r="D16" s="23">
+        <v>3</v>
+      </c>
+      <c r="F16" t="s">
+        <v>227</v>
+      </c>
+      <c r="G16" t="s">
+        <v>266</v>
+      </c>
+      <c r="H16" t="s">
+        <v>285</v>
+      </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
+      <c r="M16" t="s">
+        <v>285</v>
+      </c>
+      <c r="N16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
+      <c r="A17" t="s">
+        <v>227</v>
+      </c>
+      <c r="B17" t="s">
+        <v>266</v>
+      </c>
+      <c r="C17" t="s">
+        <v>246</v>
+      </c>
+      <c r="D17" s="23">
+        <v>1</v>
+      </c>
+      <c r="F17" t="s">
+        <v>227</v>
+      </c>
+      <c r="G17" t="s">
+        <v>266</v>
+      </c>
+      <c r="H17" t="s">
+        <v>246</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
+      </c>
+      <c r="M17" t="s">
+        <v>250</v>
+      </c>
+      <c r="N17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
+      <c r="A18" t="s">
+        <v>227</v>
+      </c>
+      <c r="B18" t="s">
+        <v>245</v>
+      </c>
+      <c r="C18" t="s">
+        <v>247</v>
+      </c>
+      <c r="D18" s="23">
+        <v>1</v>
+      </c>
+      <c r="F18" t="s">
+        <v>227</v>
+      </c>
+      <c r="G18" t="s">
+        <v>245</v>
+      </c>
+      <c r="H18" t="s">
+        <v>247</v>
+      </c>
+      <c r="I18">
+        <v>1</v>
+      </c>
+      <c r="L18" t="s">
+        <v>266</v>
+      </c>
+      <c r="M18" t="s">
+        <v>285</v>
+      </c>
+      <c r="N18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
+      <c r="A19" t="s">
+        <v>227</v>
+      </c>
+      <c r="B19" t="s">
+        <v>288</v>
+      </c>
+      <c r="C19" t="s">
+        <v>249</v>
+      </c>
+      <c r="D19" s="23">
+        <v>1</v>
+      </c>
+      <c r="F19" t="s">
+        <v>227</v>
+      </c>
+      <c r="G19" t="s">
+        <v>288</v>
+      </c>
+      <c r="H19" t="s">
+        <v>249</v>
+      </c>
+      <c r="I19">
+        <v>1</v>
+      </c>
+      <c r="L19" t="s">
+        <v>245</v>
+      </c>
+      <c r="M19" t="s">
+        <v>247</v>
+      </c>
+      <c r="N19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
+      <c r="A20" t="s">
+        <v>228</v>
+      </c>
+      <c r="B20" t="s">
+        <v>235</v>
+      </c>
+      <c r="C20" t="s">
+        <v>265</v>
+      </c>
+      <c r="D20" s="23">
+        <v>2</v>
+      </c>
+      <c r="F20" t="s">
+        <v>228</v>
+      </c>
+      <c r="G20" t="s">
+        <v>235</v>
+      </c>
+      <c r="H20" t="s">
+        <v>265</v>
+      </c>
+      <c r="I20">
+        <v>2</v>
+      </c>
+      <c r="M20" t="s">
+        <v>249</v>
+      </c>
+      <c r="N20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14">
+      <c r="A21" t="s">
+        <v>228</v>
+      </c>
+      <c r="B21" t="s">
+        <v>235</v>
+      </c>
+      <c r="C21" t="s">
+        <v>285</v>
+      </c>
+      <c r="D21" s="23">
+        <v>1</v>
+      </c>
+      <c r="F21" t="s">
+        <v>228</v>
+      </c>
+      <c r="G21" t="s">
+        <v>235</v>
+      </c>
+      <c r="H21" t="s">
+        <v>285</v>
+      </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
+      <c r="L21" t="s">
+        <v>288</v>
+      </c>
+      <c r="M21" t="s">
+        <v>249</v>
+      </c>
+      <c r="N21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14">
+      <c r="A22" t="s">
+        <v>228</v>
+      </c>
+      <c r="B22" t="s">
+        <v>235</v>
+      </c>
+      <c r="C22" t="s">
+        <v>254</v>
+      </c>
+      <c r="D22" s="23">
+        <v>2</v>
+      </c>
+      <c r="F22" t="s">
+        <v>228</v>
+      </c>
+      <c r="G22" t="s">
+        <v>235</v>
+      </c>
+      <c r="H22" t="s">
+        <v>254</v>
+      </c>
+      <c r="I22">
+        <v>2</v>
+      </c>
+      <c r="M22" t="s">
+        <v>250</v>
+      </c>
+      <c r="N22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14">
+      <c r="A23" t="s">
+        <v>228</v>
+      </c>
+      <c r="B23" t="s">
+        <v>235</v>
+      </c>
+      <c r="C23" t="s">
+        <v>236</v>
+      </c>
+      <c r="D23" s="23">
+        <v>1</v>
+      </c>
+      <c r="F23" t="s">
+        <v>228</v>
+      </c>
+      <c r="G23" t="s">
+        <v>235</v>
+      </c>
+      <c r="H23" t="s">
+        <v>236</v>
+      </c>
+      <c r="I23">
+        <v>1</v>
+      </c>
+      <c r="K23" t="s">
+        <v>228</v>
+      </c>
+      <c r="L23" t="s">
+        <v>235</v>
+      </c>
+      <c r="M23" t="s">
+        <v>235</v>
+      </c>
+      <c r="N23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14">
+      <c r="A24" t="s">
+        <v>228</v>
+      </c>
+      <c r="B24" t="s">
+        <v>235</v>
+      </c>
+      <c r="C24" t="s">
+        <v>250</v>
+      </c>
+      <c r="D24" s="23">
+        <v>1</v>
+      </c>
+      <c r="F24" t="s">
+        <v>228</v>
+      </c>
+      <c r="G24" t="s">
+        <v>235</v>
+      </c>
+      <c r="H24" t="s">
+        <v>250</v>
+      </c>
+      <c r="I24">
+        <v>1</v>
+      </c>
+      <c r="M24" t="s">
+        <v>254</v>
+      </c>
+      <c r="N24">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14">
+      <c r="A25" t="s">
+        <v>228</v>
+      </c>
+      <c r="B25" t="s">
+        <v>235</v>
+      </c>
+      <c r="C25" t="s">
+        <v>251</v>
+      </c>
+      <c r="D25" s="23">
+        <v>1</v>
+      </c>
+      <c r="F25" t="s">
+        <v>228</v>
+      </c>
+      <c r="G25" t="s">
+        <v>235</v>
+      </c>
+      <c r="H25" t="s">
+        <v>251</v>
+      </c>
+      <c r="I25">
+        <v>1</v>
+      </c>
+      <c r="M25" t="s">
+        <v>236</v>
+      </c>
+      <c r="N25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14">
+      <c r="A26" t="s">
+        <v>228</v>
+      </c>
+      <c r="B26" t="s">
+        <v>234</v>
+      </c>
+      <c r="C26" t="s">
+        <v>262</v>
+      </c>
+      <c r="D26" s="23">
+        <v>1</v>
+      </c>
+      <c r="F26" t="s">
+        <v>228</v>
+      </c>
+      <c r="G26" t="s">
+        <v>234</v>
+      </c>
+      <c r="H26" t="s">
+        <v>262</v>
+      </c>
+      <c r="I26">
+        <v>1</v>
+      </c>
+      <c r="M26" t="s">
+        <v>251</v>
+      </c>
+      <c r="N26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14">
+      <c r="A27" t="s">
+        <v>228</v>
+      </c>
+      <c r="B27" t="s">
+        <v>234</v>
+      </c>
+      <c r="C27" t="s">
+        <v>250</v>
+      </c>
+      <c r="D27" s="23">
+        <v>7</v>
+      </c>
+      <c r="F27" t="s">
+        <v>228</v>
+      </c>
+      <c r="G27" t="s">
+        <v>234</v>
+      </c>
+      <c r="H27" t="s">
+        <v>250</v>
+      </c>
+      <c r="I27">
+        <v>7</v>
+      </c>
+      <c r="L27" t="s">
+        <v>234</v>
+      </c>
+      <c r="M27" t="s">
+        <v>262</v>
+      </c>
+      <c r="N27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14">
+      <c r="A28" t="s">
+        <v>226</v>
+      </c>
+      <c r="B28" t="s">
+        <v>232</v>
+      </c>
+      <c r="C28" t="s">
+        <v>262</v>
+      </c>
+      <c r="D28" s="23">
+        <v>1</v>
+      </c>
+      <c r="F28" t="s">
+        <v>226</v>
+      </c>
+      <c r="G28" t="s">
+        <v>232</v>
+      </c>
+      <c r="H28" t="s">
+        <v>262</v>
+      </c>
+      <c r="I28">
+        <v>1</v>
+      </c>
+      <c r="M28" t="s">
+        <v>236</v>
+      </c>
+      <c r="N28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14">
+      <c r="A29" t="s">
+        <v>226</v>
+      </c>
+      <c r="B29" t="s">
+        <v>232</v>
+      </c>
+      <c r="C29" t="s">
+        <v>280</v>
+      </c>
+      <c r="D29" s="23">
+        <v>1</v>
+      </c>
+      <c r="F29" t="s">
+        <v>226</v>
+      </c>
+      <c r="G29" t="s">
+        <v>232</v>
+      </c>
+      <c r="H29" t="s">
+        <v>280</v>
+      </c>
+      <c r="I29">
+        <v>1</v>
+      </c>
+      <c r="M29" t="s">
+        <v>250</v>
+      </c>
+      <c r="N29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14">
+      <c r="A30" t="s">
+        <v>226</v>
+      </c>
+      <c r="B30" t="s">
+        <v>232</v>
+      </c>
+      <c r="C30" t="s">
+        <v>285</v>
+      </c>
+      <c r="D30" s="23">
+        <v>3</v>
+      </c>
+      <c r="F30" t="s">
+        <v>226</v>
+      </c>
+      <c r="G30" t="s">
+        <v>232</v>
+      </c>
+      <c r="H30" t="s">
+        <v>285</v>
+      </c>
+      <c r="I30">
+        <v>3</v>
+      </c>
+      <c r="M30" t="s">
+        <v>251</v>
+      </c>
+      <c r="N30">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14">
+      <c r="A31" t="s">
+        <v>226</v>
+      </c>
+      <c r="B31" t="s">
+        <v>232</v>
+      </c>
+      <c r="C31" t="s">
+        <v>241</v>
+      </c>
+      <c r="D31" s="23">
+        <v>1</v>
+      </c>
+      <c r="F31" t="s">
+        <v>226</v>
+      </c>
+      <c r="G31" t="s">
+        <v>232</v>
+      </c>
+      <c r="H31" t="s">
+        <v>241</v>
+      </c>
+      <c r="I31">
+        <v>1</v>
+      </c>
+      <c r="K31" t="s">
+        <v>226</v>
+      </c>
+      <c r="L31" t="s">
+        <v>232</v>
+      </c>
+      <c r="M31" t="s">
+        <v>262</v>
+      </c>
+      <c r="N31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14">
+      <c r="A32" t="s">
+        <v>226</v>
+      </c>
+      <c r="B32" t="s">
+        <v>232</v>
+      </c>
+      <c r="C32" t="s">
+        <v>234</v>
+      </c>
+      <c r="D32" s="23">
+        <v>1</v>
+      </c>
+      <c r="F32" t="s">
+        <v>226</v>
+      </c>
+      <c r="G32" t="s">
+        <v>232</v>
+      </c>
+      <c r="H32" t="s">
+        <v>234</v>
+      </c>
+      <c r="I32">
+        <v>1</v>
+      </c>
+      <c r="M32" t="s">
+        <v>285</v>
+      </c>
+      <c r="N32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14">
+      <c r="A33" t="s">
+        <v>226</v>
+      </c>
+      <c r="B33" t="s">
+        <v>230</v>
+      </c>
+      <c r="C33" t="s">
+        <v>262</v>
+      </c>
+      <c r="D33" s="23">
+        <v>2</v>
+      </c>
+      <c r="F33" t="s">
+        <v>226</v>
+      </c>
+      <c r="G33" t="s">
+        <v>230</v>
+      </c>
+      <c r="H33" t="s">
+        <v>262</v>
+      </c>
+      <c r="I33">
+        <v>2</v>
+      </c>
+      <c r="M33" t="s">
+        <v>241</v>
+      </c>
+      <c r="N33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14">
+      <c r="A34" t="s">
+        <v>226</v>
+      </c>
+      <c r="B34" t="s">
+        <v>230</v>
+      </c>
+      <c r="C34" t="s">
+        <v>242</v>
+      </c>
+      <c r="D34" s="23">
+        <v>2</v>
+      </c>
+      <c r="F34" t="s">
+        <v>226</v>
+      </c>
+      <c r="G34" t="s">
+        <v>230</v>
+      </c>
+      <c r="H34" t="s">
+        <v>242</v>
+      </c>
+      <c r="I34">
+        <v>2</v>
+      </c>
+      <c r="L34" t="s">
+        <v>230</v>
+      </c>
+      <c r="M34" t="s">
+        <v>262</v>
+      </c>
+      <c r="N34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14">
+      <c r="A35" t="s">
+        <v>226</v>
+      </c>
+      <c r="B35" t="s">
+        <v>230</v>
+      </c>
+      <c r="C35" t="s">
+        <v>241</v>
+      </c>
+      <c r="D35" s="23">
+        <v>3</v>
+      </c>
+      <c r="F35" t="s">
+        <v>226</v>
+      </c>
+      <c r="G35" t="s">
+        <v>230</v>
+      </c>
+      <c r="H35" t="s">
+        <v>241</v>
+      </c>
+      <c r="I35">
+        <v>3</v>
+      </c>
+      <c r="M35" t="s">
+        <v>242</v>
+      </c>
+      <c r="N35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14">
+      <c r="A36" t="s">
+        <v>226</v>
+      </c>
+      <c r="B36" t="s">
+        <v>230</v>
+      </c>
+      <c r="C36" t="s">
+        <v>267</v>
+      </c>
+      <c r="D36" s="23">
+        <v>2</v>
+      </c>
+      <c r="F36" t="s">
+        <v>226</v>
+      </c>
+      <c r="G36" t="s">
+        <v>230</v>
+      </c>
+      <c r="H36" t="s">
+        <v>267</v>
+      </c>
+      <c r="I36">
+        <v>2</v>
+      </c>
+      <c r="M36" t="s">
+        <v>241</v>
+      </c>
+      <c r="N36">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14">
+      <c r="A37" t="s">
+        <v>226</v>
+      </c>
+      <c r="B37" t="s">
+        <v>230</v>
+      </c>
+      <c r="C37" t="s">
+        <v>243</v>
+      </c>
+      <c r="D37" s="23">
+        <v>3</v>
+      </c>
+      <c r="F37" t="s">
+        <v>226</v>
+      </c>
+      <c r="G37" t="s">
+        <v>230</v>
+      </c>
+      <c r="H37" t="s">
+        <v>243</v>
+      </c>
+      <c r="I37">
+        <v>3</v>
+      </c>
+      <c r="M37" t="s">
+        <v>267</v>
+      </c>
+      <c r="N37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14">
+      <c r="A38" t="s">
+        <v>226</v>
+      </c>
+      <c r="B38" t="s">
+        <v>230</v>
+      </c>
+      <c r="C38" t="s">
+        <v>287</v>
+      </c>
+      <c r="D38" s="23">
+        <v>1</v>
+      </c>
+      <c r="F38" t="s">
+        <v>226</v>
+      </c>
+      <c r="G38" t="s">
+        <v>230</v>
+      </c>
+      <c r="H38" t="s">
+        <v>287</v>
+      </c>
+      <c r="I38">
+        <v>1</v>
+      </c>
+      <c r="M38" t="s">
+        <v>243</v>
+      </c>
+      <c r="N38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14">
+      <c r="A39" t="s">
+        <v>226</v>
+      </c>
+      <c r="B39" t="s">
+        <v>230</v>
+      </c>
+      <c r="C39" t="s">
+        <v>270</v>
+      </c>
+      <c r="D39" s="23">
+        <v>1</v>
+      </c>
+      <c r="F39" t="s">
+        <v>226</v>
+      </c>
+      <c r="G39" t="s">
+        <v>230</v>
+      </c>
+      <c r="H39" t="s">
+        <v>270</v>
+      </c>
+      <c r="I39">
+        <v>1</v>
+      </c>
+      <c r="M39" t="s">
+        <v>287</v>
+      </c>
+      <c r="N39">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14">
+      <c r="A40" t="s">
+        <v>226</v>
+      </c>
+      <c r="B40" t="s">
+        <v>231</v>
+      </c>
+      <c r="C40" t="s">
+        <v>242</v>
+      </c>
+      <c r="D40" s="23">
+        <v>1</v>
+      </c>
+      <c r="F40" t="s">
+        <v>226</v>
+      </c>
+      <c r="G40" t="s">
+        <v>231</v>
+      </c>
+      <c r="H40" t="s">
+        <v>242</v>
+      </c>
+      <c r="I40">
+        <v>1</v>
+      </c>
+      <c r="L40" t="s">
+        <v>231</v>
+      </c>
+      <c r="M40" t="s">
+        <v>262</v>
+      </c>
+      <c r="N40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14">
+      <c r="A41" t="s">
+        <v>226</v>
+      </c>
+      <c r="B41" t="s">
+        <v>231</v>
+      </c>
+      <c r="C41" t="s">
+        <v>230</v>
+      </c>
+      <c r="D41" s="23">
+        <v>1</v>
+      </c>
+      <c r="F41" t="s">
+        <v>226</v>
+      </c>
+      <c r="G41" t="s">
+        <v>231</v>
+      </c>
+      <c r="H41" t="s">
+        <v>230</v>
+      </c>
+      <c r="I41">
+        <v>1</v>
+      </c>
+      <c r="M41" t="s">
+        <v>242</v>
+      </c>
+      <c r="N41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14">
+      <c r="A42" t="s">
+        <v>226</v>
+      </c>
+      <c r="B42" t="s">
+        <v>231</v>
+      </c>
+      <c r="C42" t="s">
+        <v>241</v>
+      </c>
+      <c r="D42" s="23">
+        <v>1</v>
+      </c>
+      <c r="F42" t="s">
+        <v>226</v>
+      </c>
+      <c r="G42" t="s">
+        <v>231</v>
+      </c>
+      <c r="H42" t="s">
+        <v>241</v>
+      </c>
+      <c r="I42">
+        <v>1</v>
+      </c>
+      <c r="M42" t="s">
+        <v>241</v>
+      </c>
+      <c r="N42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14">
+      <c r="A43" t="s">
+        <v>646</v>
+      </c>
+      <c r="D43" s="23">
+        <v>80</v>
+      </c>
+      <c r="F43" t="s">
+        <v>646</v>
+      </c>
+      <c r="I43">
+        <v>80</v>
+      </c>
+      <c r="K43" t="s">
+        <v>646</v>
+      </c>
+      <c r="N43">
+        <v>80</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:T83"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="12.54296875" style="8"/>
-    <col min="2" max="2" width="129.453125" style="8" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" style="8"/>
+    <col min="2" max="2" width="129.42578125" style="8" customWidth="1"/>
     <col min="3" max="3" width="16" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.81640625" style="8" customWidth="1"/>
-    <col min="5" max="5" width="16.453125" style="8" customWidth="1"/>
-    <col min="6" max="6" width="16.81640625" style="8" customWidth="1"/>
-    <col min="7" max="7" width="15.453125" style="8" customWidth="1"/>
-    <col min="8" max="8" width="12.54296875" style="8"/>
-    <col min="9" max="9" width="255.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.453125" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="15" width="12.54296875" style="8"/>
+    <col min="4" max="4" width="15.85546875" style="8" customWidth="1"/>
+    <col min="5" max="5" width="16.42578125" style="8" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" style="8" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" style="8" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" style="8"/>
+    <col min="9" max="9" width="255.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="15" width="12.5703125" style="8"/>
     <col min="16" max="16" width="15" style="8" customWidth="1"/>
     <col min="17" max="17" width="16" style="8" customWidth="1"/>
-    <col min="18" max="18" width="15.81640625" style="8" customWidth="1"/>
-    <col min="19" max="19" width="15.7265625" style="8" customWidth="1"/>
-    <col min="20" max="20" width="15.54296875" style="8" customWidth="1"/>
+    <col min="18" max="18" width="15.85546875" style="8" customWidth="1"/>
+    <col min="19" max="19" width="15.7109375" style="8" customWidth="1"/>
+    <col min="20" max="20" width="15.5703125" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="12.5">
+    <row r="1" spans="1:20" ht="12.75">
       <c r="A1" s="12" t="s">
         <v>28</v>
       </c>
@@ -2707,7 +6377,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="12.5">
+    <row r="2" spans="1:20" ht="12.75">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2769,7 +6439,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="3" spans="1:20" ht="12.5">
+    <row r="3" spans="1:20" ht="12.75">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2831,7 +6501,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="12.5">
+    <row r="4" spans="1:20" ht="12.75">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2893,7 +6563,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="5" spans="1:20" ht="12.5">
+    <row r="5" spans="1:20" ht="12.75">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2955,8 +6625,8 @@
         <v>194</v>
       </c>
     </row>
-    <row r="6" spans="1:20" ht="12.5">
-      <c r="A6" s="22">
+    <row r="6" spans="1:20" ht="12.75">
+      <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
@@ -3017,8 +6687,8 @@
         <v>194</v>
       </c>
     </row>
-    <row r="7" spans="1:20" ht="12.5">
-      <c r="A7" s="22">
+    <row r="7" spans="1:20" ht="12.75">
+      <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
@@ -3079,8 +6749,8 @@
         <v>300</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="12.5">
-      <c r="A8" s="22">
+    <row r="8" spans="1:20" ht="12.75">
+      <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
@@ -3141,8 +6811,8 @@
         <v>194</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="12.5">
-      <c r="A9" s="22">
+    <row r="9" spans="1:20" ht="12.75">
+      <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
@@ -3203,8 +6873,8 @@
         <v>277</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="16">
-      <c r="A10" s="22">
+    <row r="10" spans="1:20" ht="14.25">
+      <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
@@ -3265,7 +6935,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="16">
+    <row r="11" spans="1:20" ht="14.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3327,7 +6997,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="12" spans="1:20" ht="16">
+    <row r="12" spans="1:20" ht="14.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -3389,7 +7059,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="13" spans="1:20" ht="16">
+    <row r="13" spans="1:20" ht="14.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -3451,7 +7121,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="14" spans="1:20" ht="16">
+    <row r="14" spans="1:20" ht="14.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3513,7 +7183,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="15" spans="1:20" ht="16">
+    <row r="15" spans="1:20" ht="14.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3575,7 +7245,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="16" spans="1:20" ht="16">
+    <row r="16" spans="1:20" ht="14.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3637,7 +7307,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="17" spans="1:20" ht="16">
+    <row r="17" spans="1:20" ht="14.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3699,7 +7369,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="18" spans="1:20" ht="16">
+    <row r="18" spans="1:20" ht="14.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3761,7 +7431,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="19" spans="1:20" ht="16">
+    <row r="19" spans="1:20" ht="14.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -3823,7 +7493,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="16">
+    <row r="20" spans="1:20" ht="14.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -3885,7 +7555,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="21" spans="1:20" ht="16">
+    <row r="21" spans="1:20" ht="14.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -3947,7 +7617,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="16">
+    <row r="22" spans="1:20" ht="14.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -4009,7 +7679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:20" ht="16">
+    <row r="23" spans="1:20" ht="14.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -4071,7 +7741,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="24" spans="1:20" ht="16">
+    <row r="24" spans="1:20" ht="14.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -4133,7 +7803,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="25" spans="1:20" ht="16">
+    <row r="25" spans="1:20" ht="14.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -4195,7 +7865,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="26" spans="1:20" ht="16">
+    <row r="26" spans="1:20" ht="14.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -4257,7 +7927,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="27" spans="1:20" ht="16">
+    <row r="27" spans="1:20" ht="14.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -4319,7 +7989,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="28" spans="1:20" ht="16">
+    <row r="28" spans="1:20" ht="14.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -4381,7 +8051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:20" ht="16">
+    <row r="29" spans="1:20" ht="14.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -4443,7 +8113,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="30" spans="1:20" ht="16">
+    <row r="30" spans="1:20" ht="14.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -4505,7 +8175,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="31" spans="1:20" ht="16">
+    <row r="31" spans="1:20" ht="14.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -4567,7 +8237,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="32" spans="1:20" ht="16">
+    <row r="32" spans="1:20" ht="14.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -4629,7 +8299,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="33" spans="1:20" ht="16">
+    <row r="33" spans="1:20" ht="14.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -4691,7 +8361,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="34" spans="1:20" ht="16">
+    <row r="34" spans="1:20" ht="14.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -4753,7 +8423,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="35" spans="1:20" ht="16">
+    <row r="35" spans="1:20" ht="14.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -4815,7 +8485,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="36" spans="1:20" ht="16">
+    <row r="36" spans="1:20" ht="14.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -4877,7 +8547,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="37" spans="1:20" ht="16">
+    <row r="37" spans="1:20" ht="14.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -4939,7 +8609,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="38" spans="1:20" ht="16">
+    <row r="38" spans="1:20" ht="14.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -5001,7 +8671,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="39" spans="1:20" ht="16">
+    <row r="39" spans="1:20" ht="14.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -5063,7 +8733,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="40" spans="1:20" ht="16">
+    <row r="40" spans="1:20" ht="14.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -5125,7 +8795,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="41" spans="1:20" ht="16">
+    <row r="41" spans="1:20" ht="14.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -5187,7 +8857,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="42" spans="1:20" ht="16">
+    <row r="42" spans="1:20" ht="14.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -5249,7 +8919,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="43" spans="1:20" ht="16">
+    <row r="43" spans="1:20" ht="14.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -5311,7 +8981,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="44" spans="1:20" ht="16">
+    <row r="44" spans="1:20" ht="14.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -5373,7 +9043,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="45" spans="1:20" ht="16">
+    <row r="45" spans="1:20" ht="14.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -5435,7 +9105,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="46" spans="1:20" ht="16">
+    <row r="46" spans="1:20" ht="14.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -5497,7 +9167,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="47" spans="1:20" ht="16">
+    <row r="47" spans="1:20" ht="14.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -5559,7 +9229,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="48" spans="1:20" ht="16">
+    <row r="48" spans="1:20" ht="14.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -5621,7 +9291,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="49" spans="1:20" ht="16">
+    <row r="49" spans="1:20" ht="14.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -5683,7 +9353,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="50" spans="1:20" ht="16">
+    <row r="50" spans="1:20" ht="14.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -5745,7 +9415,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="51" spans="1:20" ht="16">
+    <row r="51" spans="1:20" ht="14.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -5807,7 +9477,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="52" spans="1:20" ht="16">
+    <row r="52" spans="1:20" ht="14.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -5869,7 +9539,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="53" spans="1:20" ht="16">
+    <row r="53" spans="1:20" ht="14.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -5931,7 +9601,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="54" spans="1:20" ht="16">
+    <row r="54" spans="1:20" ht="14.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -5993,7 +9663,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="55" spans="1:20" ht="16">
+    <row r="55" spans="1:20" ht="14.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -6055,7 +9725,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="56" spans="1:20" ht="16">
+    <row r="56" spans="1:20" ht="14.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -6117,7 +9787,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="57" spans="1:20" ht="16">
+    <row r="57" spans="1:20" ht="14.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -6179,7 +9849,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="58" spans="1:20" ht="16">
+    <row r="58" spans="1:20" ht="14.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -6241,7 +9911,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="59" spans="1:20" ht="16">
+    <row r="59" spans="1:20" ht="14.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -6303,7 +9973,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="60" spans="1:20" ht="16">
+    <row r="60" spans="1:20" ht="14.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -6365,7 +10035,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="61" spans="1:20" ht="16">
+    <row r="61" spans="1:20" ht="14.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -6427,7 +10097,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="62" spans="1:20" ht="16">
+    <row r="62" spans="1:20" ht="14.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -6489,7 +10159,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="63" spans="1:20" ht="16">
+    <row r="63" spans="1:20" ht="14.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -6551,7 +10221,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="64" spans="1:20" ht="16">
+    <row r="64" spans="1:20" ht="14.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -6613,7 +10283,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="65" spans="1:20" ht="16">
+    <row r="65" spans="1:20" ht="14.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -6675,7 +10345,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="66" spans="1:20" ht="16">
+    <row r="66" spans="1:20" ht="14.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -6737,7 +10407,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="67" spans="1:20" ht="16">
+    <row r="67" spans="1:20" ht="14.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -6799,7 +10469,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="68" spans="1:20" ht="16">
+    <row r="68" spans="1:20" ht="14.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -6861,7 +10531,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="69" spans="1:20" ht="16">
+    <row r="69" spans="1:20" ht="14.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -6923,7 +10593,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="70" spans="1:20" ht="16">
+    <row r="70" spans="1:20" ht="14.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -6985,7 +10655,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="71" spans="1:20" ht="12.5">
+    <row r="71" spans="1:20" ht="12.75">
       <c r="A71">
         <v>70</v>
       </c>
@@ -7047,7 +10717,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="72" spans="1:20" ht="12.5">
+    <row r="72" spans="1:20" ht="12.75">
       <c r="A72">
         <v>71</v>
       </c>
@@ -7109,7 +10779,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="73" spans="1:20" ht="12.5">
+    <row r="73" spans="1:20" ht="12.75">
       <c r="A73">
         <v>72</v>
       </c>
@@ -7171,7 +10841,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="74" spans="1:20" ht="12.5">
+    <row r="74" spans="1:20" ht="12.75">
       <c r="A74">
         <v>73</v>
       </c>
@@ -7233,7 +10903,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="75" spans="1:20" ht="12.5">
+    <row r="75" spans="1:20" ht="12.75">
       <c r="A75">
         <v>74</v>
       </c>
@@ -7295,7 +10965,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="76" spans="1:20" ht="12.5">
+    <row r="76" spans="1:20" ht="12.75">
       <c r="A76">
         <v>75</v>
       </c>
@@ -7357,7 +11027,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="77" spans="1:20" ht="12.5">
+    <row r="77" spans="1:20" ht="12.75">
       <c r="A77">
         <v>76</v>
       </c>
@@ -7419,7 +11089,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="78" spans="1:20" ht="12.5">
+    <row r="78" spans="1:20" ht="12.75">
       <c r="A78">
         <v>77</v>
       </c>
@@ -7481,7 +11151,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="79" spans="1:20" ht="12.5">
+    <row r="79" spans="1:20" ht="12.75">
       <c r="A79">
         <v>78</v>
       </c>
@@ -7543,7 +11213,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="80" spans="1:20" ht="12.5">
+    <row r="80" spans="1:20" ht="12.75">
       <c r="A80">
         <v>79</v>
       </c>
@@ -7605,7 +11275,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="81" spans="1:20" ht="12.5">
+    <row r="81" spans="1:20" ht="12.75">
       <c r="A81">
         <v>80</v>
       </c>
@@ -7667,7 +11337,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="82" spans="1:20" ht="12.5">
+    <row r="82" spans="1:20" ht="12.75">
       <c r="B82" s="7"/>
       <c r="C82" s="7"/>
       <c r="D82" s="7"/>
@@ -7675,7 +11345,7 @@
       <c r="L82" s="7"/>
       <c r="P82" s="7"/>
     </row>
-    <row r="83" spans="1:20" ht="12.5">
+    <row r="83" spans="1:20" ht="12.75">
       <c r="B83" s="7"/>
       <c r="C83" s="7"/>
       <c r="D83" s="7"/>
@@ -7685,31 +11355,31 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:T81" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="B37">
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B82:B1048576 B1">
-    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B37">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32DFED4D-37E4-4DCB-B19D-D2AFCC6828E3}">
   <dimension ref="A1:L82"/>
-  <sheetFormatPr defaultRowHeight="12.5"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="175.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="255.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="24.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="28.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="24.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="175.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="255.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="24.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -9118,7 +12788,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="38" spans="1:12" ht="16">
+    <row r="38" spans="1:12" ht="14.25">
       <c r="A38" s="21">
         <v>37</v>
       </c>
@@ -10836,10 +14506,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7B2B4AC-AA3E-486F-AA22-B5E796120EA1}">
   <dimension ref="A1:T41"/>
-  <sheetFormatPr defaultRowHeight="12.5"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" t="s">
@@ -13388,15 +17058,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28B9ABF6-17D7-457F-8305-77AF789C31D2}">
   <dimension ref="A1:A83"/>
-  <sheetFormatPr defaultRowHeight="12.5"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="26.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="25">
+    <row r="1" spans="1:1" ht="25.5">
       <c r="A1" s="19" t="s">
         <v>222</v>
       </c>
@@ -13421,7 +17091,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="25">
+    <row r="6" spans="1:1" ht="25.5">
       <c r="A6" s="19" t="s">
         <v>223</v>
       </c>
@@ -13521,7 +17191,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="26" spans="1:1" ht="25">
+    <row r="26" spans="1:1" ht="25.5">
       <c r="A26" s="19" t="s">
         <v>224</v>
       </c>
@@ -13681,7 +17351,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="58" spans="1:1" ht="25">
+    <row r="58" spans="1:1" ht="25.5">
       <c r="A58" s="19" t="s">
         <v>225</v>
       </c>
@@ -13820,12 +17490,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1A6D6A6-C2D9-4142-8A18-4A685F878828}">
   <dimension ref="A1:E61"/>
-  <sheetFormatPr defaultRowHeight="12.5"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -14870,13 +18540,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BB95410-4578-451E-AEA9-509ABC9E23A6}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="12.5"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>